<commit_message>
Animations vendeurs +  update sprint + test model Client
Update stand
</commit_message>
<xml_diff>
--- a/Journal_de_sprint.xlsx
+++ b/Journal_de_sprint.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bdebqcca-my.sharepoint.com/personal/2239437_bdeb_qc_ca/Documents/Documents/GitHub Unity/Horaire 0.9/Horaire-0.9/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2281126\Documents\GitHub\projet-de-session-5gd-a25-gr-e\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="13_ncr:1_{8E34BB9D-75EF-421A-B832-2F348A795421}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E8C823E6-2FBB-40E2-9626-787DA430104C}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86B4CEA7-30C1-4FFA-B23E-45EF529F74A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6BF6013A-4C68-4CEF-BF49-8F7071437FDB}"/>
   </bookViews>
@@ -102,7 +102,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="56">
   <si>
     <t>Item planifié</t>
   </si>
@@ -128,9 +128,6 @@
     <t>S'authentifier avec son compte usager</t>
   </si>
   <si>
-    <t>ETQ usager, je veux créer mon compte pou raccéder aux fonctions du site</t>
-  </si>
-  <si>
     <t>Récit</t>
   </si>
   <si>
@@ -140,43 +137,13 @@
     <t>Jacques</t>
   </si>
   <si>
-    <t>X</t>
-  </si>
-  <si>
     <t>Tâche</t>
   </si>
   <si>
-    <t>Créer la BD des comptes usagers</t>
-  </si>
-  <si>
-    <t>Créer la page d'inscription</t>
-  </si>
-  <si>
-    <t>Valider l'inscription en double</t>
-  </si>
-  <si>
-    <t>Procéder à l'inscription (validation, hachage)</t>
-  </si>
-  <si>
     <t>Guillaume</t>
   </si>
   <si>
     <t>Aurèle</t>
-  </si>
-  <si>
-    <t>Saga</t>
-  </si>
-  <si>
-    <t>Gérer les comptes utilisateurs</t>
-  </si>
-  <si>
-    <t>Créer la page de login</t>
-  </si>
-  <si>
-    <t>Valider les données d'authentification</t>
-  </si>
-  <si>
-    <t>ETQ usager, je veux m'authentifier comme membre du site</t>
   </si>
   <si>
     <t>Temps de cycle moyen (récits)</t>
@@ -351,12 +318,48 @@
   <si>
     <t>-</t>
   </si>
+  <si>
+    <t>Création de l’interface de base</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Barre de score de réputation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Barre d’argent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Setup de la NavMesh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Creation du script de mouvement des agents</t>
+  </si>
+  <si>
+    <t>Fonctionnement des agents</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Setup des NavMeshObstacles</t>
+  </si>
+  <si>
+    <t>Animations</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Animation du vendeur de poisson</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Animation du vendeur d'armes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Setup du magasin du joueur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -413,6 +416,19 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF3F3F76"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -504,15 +520,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="3" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -538,6 +545,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="3" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -915,17 +927,17 @@
       <c r="G1" s="18"/>
       <c r="H1" s="18"/>
       <c r="I1" s="18"/>
-      <c r="K1" s="13" t="s">
+      <c r="K1" s="10" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="K2" t="s">
-        <v>25</v>
-      </c>
-      <c r="L2" s="9">
+        <v>14</v>
+      </c>
+      <c r="L2" s="6" t="e">
         <f>AVERAGEIFS(H:H,G:G, "X", B:B, "Récit")</f>
-        <v>4</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -933,19 +945,19 @@
         <v>0</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>1</v>
@@ -957,308 +969,347 @@
         <v>6</v>
       </c>
       <c r="K3" t="s">
-        <v>26</v>
-      </c>
-      <c r="L3" s="9">
+        <v>15</v>
+      </c>
+      <c r="L3" s="6" t="e">
         <f>AVERAGEIFS(H:H,G:G, "X", B:B, "Tâche")</f>
-        <v>1.8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" s="6" t="s">
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="K4" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-      <c r="K4" t="s">
-        <v>31</v>
-      </c>
-      <c r="L4" s="9">
+      <c r="L4" s="6">
         <f>COUNTIFS(G:G, "X", B:B, "Récit")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="7">
-        <v>0.5</v>
-      </c>
-      <c r="D5" s="7">
-        <v>0.4</v>
-      </c>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7">
-        <v>0.1</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>12</v>
-      </c>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="3"/>
       <c r="H5" s="1">
         <v>4</v>
       </c>
       <c r="I5" s="1"/>
       <c r="K5" t="s">
-        <v>32</v>
-      </c>
-      <c r="L5" s="9">
+        <v>21</v>
+      </c>
+      <c r="L5" s="6">
         <f>COUNTIFS(G:G, "X", B:B, "Tâche")</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7">
-        <v>1</v>
-      </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="6" t="s">
-        <v>12</v>
-      </c>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="3"/>
       <c r="H6" s="1">
         <v>1</v>
       </c>
       <c r="I6" s="1"/>
     </row>
-    <row r="7" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="7">
-        <v>0.8</v>
-      </c>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7">
-        <v>0.2</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>12</v>
-      </c>
+    <row r="7" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="3"/>
       <c r="H7" s="1">
         <v>2</v>
       </c>
       <c r="I7" s="1"/>
-      <c r="K7" s="14" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7">
-        <v>0.75</v>
-      </c>
-      <c r="F8" s="7">
-        <v>0.25</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>12</v>
-      </c>
+      <c r="K7" s="11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4">
+        <v>1</v>
+      </c>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="3"/>
       <c r="H8" s="1">
         <v>1</v>
       </c>
       <c r="I8" s="1"/>
       <c r="K8" t="s">
-        <v>28</v>
-      </c>
-      <c r="L8" s="9">
+        <v>17</v>
+      </c>
+      <c r="L8" s="6">
         <f>COUNTIF(B:B,"Récit")</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="7">
-        <v>1</v>
-      </c>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="6" t="s">
-        <v>12</v>
-      </c>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4">
+        <v>0.25</v>
+      </c>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="3"/>
       <c r="H9" s="1">
         <v>3</v>
       </c>
       <c r="I9" s="1"/>
       <c r="K9" t="s">
-        <v>29</v>
-      </c>
-      <c r="L9" s="9">
+        <v>18</v>
+      </c>
+      <c r="L9" s="6">
         <f>COUNTIF(B:B, "Tâche")</f>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4">
         <v>1</v>
       </c>
-      <c r="F10" s="7"/>
-      <c r="G10" s="6"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="3"/>
       <c r="H10" s="1"/>
       <c r="I10" s="1">
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="6"/>
+    <row r="11" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="4">
+        <v>0.45</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="3"/>
       <c r="H11" s="1"/>
       <c r="I11" s="1">
         <v>4</v>
       </c>
       <c r="K11" t="s">
-        <v>27</v>
-      </c>
-      <c r="L11" s="10">
+        <v>16</v>
+      </c>
+      <c r="L11" s="7">
         <f>L4/L8</f>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7">
-        <v>0.5</v>
-      </c>
-      <c r="E12" s="7">
-        <v>0.5</v>
-      </c>
-      <c r="F12" s="7"/>
-      <c r="G12" s="6" t="s">
-        <v>12</v>
-      </c>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="3"/>
       <c r="H12" s="1">
         <v>2</v>
       </c>
       <c r="I12" s="1"/>
       <c r="K12" t="s">
-        <v>30</v>
-      </c>
-      <c r="L12" s="10">
+        <v>19</v>
+      </c>
+      <c r="L12" s="7">
         <f>L5/L9</f>
-        <v>0.83333333333333337</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="K14" s="14" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="1">
+        <v>2</v>
+      </c>
+      <c r="I13" s="1"/>
+    </row>
+    <row r="14" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" s="4">
+        <v>1</v>
+      </c>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="1">
+        <v>3</v>
+      </c>
+      <c r="I14" s="1"/>
+      <c r="K14" s="11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="16"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
       <c r="K15" t="s">
+        <v>9</v>
+      </c>
+      <c r="L15" s="6">
+        <f>SUMIFS(C:C,G:G,"X")</f>
+        <v>0</v>
+      </c>
+      <c r="M15" s="7" t="e">
+        <f>L15/SUM($L$15:$L$18)</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" s="3"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="K16" t="s">
+        <v>12</v>
+      </c>
+      <c r="L16" s="6">
+        <f>SUMIFS(D:D,G:G,"X")</f>
+        <v>0</v>
+      </c>
+      <c r="M16" s="7" t="e">
+        <f>L16/SUM($L$15:$L$18)</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="16"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="K17" t="s">
         <v>10</v>
       </c>
-      <c r="L15" s="9">
-        <f>SUMIFS(C:C,G:G,"X")</f>
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="M15" s="10">
-        <f>L15/SUM($L$15:$L$18)</f>
-        <v>0.38333333333333336</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="K16" t="s">
-        <v>18</v>
-      </c>
-      <c r="L16" s="9">
-        <f>SUMIFS(D:D,G:G,"X")</f>
-        <v>1.9</v>
-      </c>
-      <c r="M16" s="10">
-        <f>L16/SUM($L$15:$L$18)</f>
-        <v>0.31666666666666671</v>
-      </c>
-    </row>
-    <row r="17" spans="11:15" x14ac:dyDescent="0.25">
-      <c r="K17" t="s">
-        <v>11</v>
-      </c>
-      <c r="L17" s="9">
+      <c r="L17" s="6">
         <f>SUMIFS(E:E,G:G,"X")</f>
-        <v>1.25</v>
-      </c>
-      <c r="M17" s="10">
+        <v>0</v>
+      </c>
+      <c r="M17" s="7" t="e">
         <f>L17/SUM($L$15:$L$18)</f>
-        <v>0.20833333333333337</v>
-      </c>
-    </row>
-    <row r="18" spans="11:15" x14ac:dyDescent="0.25">
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="K18" t="s">
-        <v>19</v>
-      </c>
-      <c r="L18" s="9">
+        <v>13</v>
+      </c>
+      <c r="L18" s="6">
         <f>SUMIFS(F:F,G:G,"X")</f>
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="M18" s="10">
+        <v>0</v>
+      </c>
+      <c r="M18" s="7" t="e">
         <f>L18/SUM($L$15:$L$18)</f>
-        <v>9.1666666666666688E-2</v>
-      </c>
-    </row>
-    <row r="20" spans="11:15" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="K20" s="13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="21" spans="11:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" ht="18" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="K20" s="10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="L21" s="19" t="s">
         <v>4</v>
       </c>
@@ -1266,9 +1317,9 @@
       <c r="N21" s="19"/>
       <c r="O21" s="19"/>
     </row>
-    <row r="22" spans="11:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="K22" s="14" t="s">
-        <v>37</v>
+    <row r="22" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K22" s="11" t="s">
+        <v>26</v>
       </c>
       <c r="L22">
         <v>1</v>
@@ -1283,63 +1334,63 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="11:15" ht="127.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K23" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="L23" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="M23" s="11"/>
-      <c r="N23" s="11"/>
-      <c r="O23" s="11"/>
-    </row>
-    <row r="24" spans="11:15" ht="123.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K24" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="L24" s="15" t="s">
+    <row r="23" spans="1:15" ht="127.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K23" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="L23" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="M23" s="8"/>
+      <c r="N23" s="8"/>
+      <c r="O23" s="8"/>
+    </row>
+    <row r="24" spans="1:15" ht="123.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K24" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="L24" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="M24" s="8"/>
+      <c r="N24" s="8"/>
+      <c r="O24" s="8"/>
+    </row>
+    <row r="25" spans="1:15" ht="117.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K25" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="M24" s="11"/>
-      <c r="N24" s="11"/>
-      <c r="O24" s="11"/>
-    </row>
-    <row r="25" spans="11:15" ht="117.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K25" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="L25" s="11"/>
-      <c r="M25" s="11"/>
-      <c r="N25" s="11"/>
-      <c r="O25" s="11"/>
-    </row>
-    <row r="26" spans="11:15" ht="101.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K26" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="L26" s="12"/>
-      <c r="M26" s="12"/>
-      <c r="N26" s="12"/>
-      <c r="O26" s="12"/>
-    </row>
-    <row r="30" spans="11:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="K30" s="14" t="s">
+      <c r="L25" s="8"/>
+      <c r="M25" s="8"/>
+      <c r="N25" s="8"/>
+      <c r="O25" s="8"/>
+    </row>
+    <row r="26" spans="1:15" ht="101.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K26" s="13" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="31" spans="11:15" ht="44.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K31" s="16" t="s">
-        <v>40</v>
+      <c r="L26" s="9"/>
+      <c r="M26" s="9"/>
+      <c r="N26" s="9"/>
+      <c r="O26" s="9"/>
+    </row>
+    <row r="30" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K30" s="11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" ht="44.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K31" s="13" t="s">
+        <v>29</v>
       </c>
       <c r="L31" s="20"/>
       <c r="M31" s="20"/>
       <c r="N31" s="20"/>
       <c r="O31" s="20"/>
     </row>
-    <row r="32" spans="11:15" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K32" s="16" t="s">
-        <v>41</v>
+    <row r="32" spans="1:15" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K32" s="13" t="s">
+        <v>30</v>
       </c>
       <c r="L32" s="17"/>
       <c r="M32" s="17"/>
@@ -1347,13 +1398,13 @@
       <c r="O32" s="17"/>
     </row>
     <row r="34" spans="11:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="K34" s="14" t="s">
-        <v>42</v>
+      <c r="K34" s="11" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="35" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K35" s="16" t="s">
-        <v>43</v>
+      <c r="K35" s="13" t="s">
+        <v>32</v>
       </c>
       <c r="L35" s="17"/>
       <c r="M35" s="17"/>
@@ -1361,8 +1412,8 @@
       <c r="O35" s="17"/>
     </row>
     <row r="36" spans="11:15" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K36" s="16" t="s">
-        <v>44</v>
+      <c r="K36" s="13" t="s">
+        <v>33</v>
       </c>
       <c r="L36" s="17"/>
       <c r="M36" s="17"/>
@@ -1370,8 +1421,8 @@
       <c r="O36" s="17"/>
     </row>
     <row r="37" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K37" s="16" t="s">
-        <v>45</v>
+      <c r="K37" s="13" t="s">
+        <v>34</v>
       </c>
       <c r="L37" s="17"/>
       <c r="M37" s="17"/>
@@ -1379,15 +1430,15 @@
       <c r="O37" s="17"/>
     </row>
     <row r="38" spans="11:15" x14ac:dyDescent="0.25">
-      <c r="K38" s="16"/>
-      <c r="L38" s="16"/>
-      <c r="M38" s="16"/>
-      <c r="N38" s="16"/>
-      <c r="O38" s="16"/>
+      <c r="K38" s="13"/>
+      <c r="L38" s="13"/>
+      <c r="M38" s="13"/>
+      <c r="N38" s="13"/>
+      <c r="O38" s="13"/>
     </row>
     <row r="39" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K39" s="16" t="s">
-        <v>46</v>
+      <c r="K39" s="13" t="s">
+        <v>35</v>
       </c>
       <c r="L39" s="17"/>
       <c r="M39" s="17"/>
@@ -1406,7 +1457,7 @@
     <mergeCell ref="L32:O32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Sprint (avec Émile)
Contribution des deux coéquipiers sur les Sprints d'équipe
</commit_message>
<xml_diff>
--- a/Journal_de_sprint.xlsx
+++ b/Journal_de_sprint.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2281126\Documents\GitHub\projet-de-session-5gd-a25-gr-e\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66D0A666-8AB5-4380-8E33-DF6A4E43F1C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8B74B68-E30C-4B73-A8C4-50462ED4F44C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{6BF6013A-4C68-4CEF-BF49-8F7071437FDB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{6BF6013A-4C68-4CEF-BF49-8F7071437FDB}"/>
   </bookViews>
   <sheets>
-    <sheet name="Exemple" sheetId="1" r:id="rId1"/>
-    <sheet name="Exemple (2)" sheetId="2" r:id="rId2"/>
+    <sheet name="Sprint1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sprint2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sprint3" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -168,8 +169,74 @@
 </comments>
 </file>
 
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Stéphane Lévesque</author>
+  </authors>
+  <commentList>
+    <comment ref="B3" authorId="0" shapeId="0" xr:uid="{2D2E4ED3-38E9-4079-8854-EB420CC832F1}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Utiliser:
+Saga pour un ensemble de récits
+Récit pour une fonction du point de vue de son usager
+Tâche pour l'implantation d'une partie d'un récit, une correction de bug ou tout autre travail technique de nature non-fonctionnelle.
+Respecter l'orthographe exact (majuscules et accents)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G3" authorId="0" shapeId="0" xr:uid="{B713B9E9-E707-4DE1-AC68-01F7B1C0515A}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Indiquer X (majuscule) si l'item est conforme à la Définition de Terminé</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H3" authorId="0" shapeId="0" xr:uid="{F5D980EA-2B07-4BB8-92B6-EF444F3FFE95}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Le nombre de jours entre le début et la fin du travail sur cet item (minimum 1)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I3" authorId="0" shapeId="0" xr:uid="{5AAC720F-4F57-4AF8-B8E8-633026B74B70}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Nombre de jours depuis le début du travail sur cet item (minimum 1)</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="77">
   <si>
     <t>Item planifié</t>
   </si>
@@ -198,21 +265,9 @@
     <t>Récit</t>
   </si>
   <si>
-    <t>Joseph</t>
-  </si>
-  <si>
-    <t>Jacques</t>
-  </si>
-  <si>
     <t>Tâche</t>
   </si>
   <si>
-    <t>Guillaume</t>
-  </si>
-  <si>
-    <t>Aurèle</t>
-  </si>
-  <si>
     <t>Temps de cycle moyen (récits)</t>
   </si>
   <si>
@@ -283,12 +338,6 @@
   </si>
   <si>
     <t>Membre 2</t>
-  </si>
-  <si>
-    <t>Membre 3</t>
-  </si>
-  <si>
-    <t>Membre 4</t>
   </si>
   <si>
     <r>
@@ -386,47 +435,252 @@
     <t>-</t>
   </si>
   <si>
-    <t>Création de l’interface de base</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Barre de score de réputation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Barre d’argent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Setup de la NavMesh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Creation du script de mouvement des agents</t>
-  </si>
-  <si>
-    <t>Fonctionnement des agents</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Setup des NavMeshObstacles</t>
-  </si>
-  <si>
-    <t>Animations</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Animation du vendeur de poisson</t>
   </si>
   <si>
     <t xml:space="preserve"> Animation du vendeur d'armes</t>
   </si>
   <si>
-    <t xml:space="preserve">  Setup du magasin du joueur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  </t>
+    <t>Saga</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mise en place </t>
+  </si>
+  <si>
+    <t>Avoir un projet Unity fonctionnel afin de commencer le développement</t>
+  </si>
+  <si>
+    <t>Base visuelle et environnement</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Avoir un marché médiéval de base</t>
+  </si>
+  <si>
+    <t>Prototype UI</t>
+  </si>
+  <si>
+    <t>Hiérarchie d'interface de base</t>
+  </si>
+  <si>
+    <t>Prototype PNJ</t>
+  </si>
+  <si>
+    <t>Avoir une NavMesh et des agents fonctionels</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Importation de la scène Low-Poly Medieval Market de base</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Ajout de colliders de base sur la map</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Ajout d’un gitignore adapté Unity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Organisation initiale du dépôt et des dossiers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Création d’un Canvas </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  TextMeshPro basique pour le compteur de pièces</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Importation TextMeshPro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Création du repo GitHub + projet Unity </t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Ajout des NavMeshObstacles et Bake</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Ajout d'un agent pour test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Creation d'un script "Wandering" pour le mouvement aléatoire</t>
+  </si>
+  <si>
+    <t>Stabilisation et organisation du projet</t>
+  </si>
+  <si>
+    <t>Dépôt bien organisé et fonctionnel afin d’éviter les conflits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Réorganisation dossiers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Séparation des assets / scènes </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Correction du .gitignore pour éviter push de gros fichiers </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Migration Unity (2022 → 6000) et compatibilité </t>
+  </si>
+  <si>
+    <t>Decoration visuelle du magasin du joueur</t>
+  </si>
+  <si>
+    <t>Decoration du magasin pour mieux comprendre le role du vendeur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Placement d’objets (livres, fioles, baguettes, boule de cristal)</t>
+  </si>
+  <si>
+    <t>Animation des magasins</t>
+  </si>
+  <si>
+    <t>Avoir des animations pour rendre le marche plus vivant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Animations du PNJ "Mushroom Man"</t>
+  </si>
+  <si>
+    <t>Émile</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Progrès accomplis:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Travail Sprint.                   </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Objectifs pour la journée : Finir Sprint1 et Sprint2 equipe e</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">t pull Git            </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Obstacles rencontrés:Erreurs de build des packages Unity</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Progrès accomplis:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Travail Sprint.                   </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Objectifs pour la journée : Finir Sprint1 et Sprint2 equipe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.            </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Obstacles rencontrés:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Memorisation de l'ordre des tâches.                                           </t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -500,6 +754,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -519,7 +780,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -564,13 +825,37 @@
       <left style="thin">
         <color rgb="FF7F7F7F"/>
       </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
         <color rgb="FF7F7F7F"/>
       </right>
       <top style="thin">
         <color rgb="FF7F7F7F"/>
       </top>
-      <bottom/>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -581,7 +866,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="3"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -601,9 +886,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="3" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="2"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="3" applyAlignment="1">
@@ -612,11 +894,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="3" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="3" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="3" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -624,9 +909,16 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="3" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Calcul" xfId="4" builtinId="22"/>
@@ -968,7 +1260,7 @@
   <dimension ref="A1:O39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="66.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="67.5703125" customWidth="1"/>
     <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="6" width="10.28515625" customWidth="1"/>
     <col min="7" max="7" width="8.140625" style="2" bestFit="1" customWidth="1"/>
@@ -994,17 +1286,17 @@
       <c r="G1" s="18"/>
       <c r="H1" s="18"/>
       <c r="I1" s="18"/>
-      <c r="K1" s="10" t="s">
+      <c r="K1" s="9" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="K2" t="s">
-        <v>14</v>
-      </c>
-      <c r="L2" s="6" t="e">
+        <v>10</v>
+      </c>
+      <c r="L2" s="6">
         <f>AVERAGEIFS(H:H,G:G, "X", B:B, "Récit")</f>
-        <v>#DIV/0!</v>
+        <v>1.3333333333333333</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -1012,19 +1304,19 @@
         <v>0</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>1</v>
@@ -1036,19 +1328,19 @@
         <v>6</v>
       </c>
       <c r="K3" t="s">
-        <v>15</v>
-      </c>
-      <c r="L3" s="6" t="e">
+        <v>11</v>
+      </c>
+      <c r="L3" s="6">
         <f>AVERAGEIFS(H:H,G:G, "X", B:B, "Tâche")</f>
-        <v>#DIV/0!</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
@@ -1058,325 +1350,401 @@
       <c r="H4" s="5"/>
       <c r="I4" s="5"/>
       <c r="K4" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="L4" s="6">
         <f>COUNTIFS(G:G, "X", B:B, "Récit")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
-        <v>45</v>
+      <c r="A5" s="14" t="s">
+        <v>42</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
-      <c r="G5" s="3"/>
+      <c r="G5" s="3" t="s">
+        <v>58</v>
+      </c>
       <c r="H5" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I5" s="1"/>
       <c r="K5" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="L5" s="6">
         <f>COUNTIFS(G:G, "X", B:B, "Tâche")</f>
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
-        <v>46</v>
+      <c r="A6" s="14" t="s">
+        <v>57</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="4">
-        <v>0.1</v>
-      </c>
-      <c r="D6" s="4"/>
+        <v>9</v>
+      </c>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4">
+        <v>1</v>
+      </c>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
-      <c r="G6" s="3"/>
+      <c r="G6" s="3" t="s">
+        <v>44</v>
+      </c>
       <c r="H6" s="1">
         <v>1</v>
       </c>
       <c r="I6" s="1"/>
     </row>
     <row r="7" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="16" t="s">
-        <v>49</v>
+      <c r="A7" s="14" t="s">
+        <v>52</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
+        <v>9</v>
+      </c>
+      <c r="C7" s="4">
+        <v>0.4</v>
+      </c>
+      <c r="D7" s="4">
+        <v>0.6</v>
+      </c>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
-      <c r="G7" s="3"/>
+      <c r="G7" s="3" t="s">
+        <v>44</v>
+      </c>
       <c r="H7" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I7" s="1"/>
-      <c r="K7" s="11" t="s">
-        <v>24</v>
+      <c r="K7" s="10" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="16" t="s">
-        <v>47</v>
+      <c r="A8" s="14" t="s">
+        <v>53</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="4"/>
+        <v>9</v>
+      </c>
+      <c r="C8" s="4">
+        <v>0.9</v>
+      </c>
       <c r="D8" s="4">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
-      <c r="G8" s="3"/>
+      <c r="G8" s="3" t="s">
+        <v>44</v>
+      </c>
       <c r="H8" s="1">
         <v>1</v>
       </c>
       <c r="I8" s="1"/>
       <c r="K8" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="L8" s="6">
         <f>COUNTIF(B:B,"Récit")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="16" t="s">
-        <v>48</v>
+      <c r="A9" s="14" t="s">
+        <v>43</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="C9" s="4"/>
-      <c r="D9" s="4">
-        <v>0.25</v>
-      </c>
+      <c r="D9" s="4"/>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="3"/>
-      <c r="H9" s="1">
-        <v>3</v>
-      </c>
+      <c r="H9" s="1"/>
       <c r="I9" s="1"/>
       <c r="K9" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="L9" s="6">
         <f>COUNTIF(B:B, "Tâche")</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>11</v>
-      </c>
       <c r="C10" s="4"/>
-      <c r="D10" s="4">
-        <v>1</v>
-      </c>
+      <c r="D10" s="4"/>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1">
-        <v>5</v>
-      </c>
+      <c r="G10" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H10" s="1">
+        <v>2</v>
+      </c>
+      <c r="I10" s="1"/>
     </row>
     <row r="11" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="16" t="s">
-        <v>54</v>
+      <c r="A11" s="14" t="s">
+        <v>50</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C11" s="4">
-        <v>0.45</v>
-      </c>
-      <c r="D11" s="4"/>
+        <v>9</v>
+      </c>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4">
+        <v>1</v>
+      </c>
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1">
-        <v>4</v>
-      </c>
+      <c r="G11" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H11" s="1">
+        <v>1</v>
+      </c>
+      <c r="I11" s="1"/>
       <c r="K11" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="L11" s="7">
         <f>L4/L8</f>
-        <v>0</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="16" t="s">
+      <c r="A12" s="14" t="s">
         <v>51</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
+      <c r="D12" s="4">
+        <v>1</v>
+      </c>
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
-      <c r="G12" s="3"/>
+      <c r="G12" s="3" t="s">
+        <v>44</v>
+      </c>
       <c r="H12" s="1">
         <v>2</v>
       </c>
       <c r="I12" s="1"/>
       <c r="K12" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L12" s="7">
         <f>L5/L9</f>
-        <v>0</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="16" t="s">
-        <v>52</v>
+      <c r="A13" s="14" t="s">
+        <v>46</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C13" s="4">
-        <v>0.5</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="C13" s="4"/>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
       <c r="G13" s="3"/>
-      <c r="H13" s="1">
-        <v>2</v>
-      </c>
+      <c r="H13" s="1"/>
       <c r="I13" s="1"/>
     </row>
     <row r="14" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="16" t="s">
-        <v>53</v>
+      <c r="A14" s="14" t="s">
+        <v>47</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C14" s="4">
-        <v>1</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="C14" s="4"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
-      <c r="G14" s="3"/>
+      <c r="G14" s="3" t="s">
+        <v>58</v>
+      </c>
       <c r="H14" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I14" s="1"/>
-      <c r="K14" s="11" t="s">
-        <v>22</v>
+      <c r="K14" s="10" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="16"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="4"/>
+      <c r="A15" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="4">
+        <v>1</v>
+      </c>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="1"/>
+      <c r="G15" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H15" s="1">
+        <v>1</v>
+      </c>
       <c r="I15" s="1"/>
       <c r="K15" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="L15" s="6">
         <f>SUMIFS(C:C,G:G,"X")</f>
-        <v>0</v>
-      </c>
-      <c r="M15" s="7" t="e">
+        <v>4.3</v>
+      </c>
+      <c r="M15" s="7">
         <f>L15/SUM($L$15:$L$18)</f>
-        <v>#DIV/0!</v>
+        <v>0.53749999999999998</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="B16" s="3"/>
-      <c r="C16" s="4"/>
+      <c r="A16" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" s="4">
+        <v>1</v>
+      </c>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="1"/>
+      <c r="G16" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H16" s="1">
+        <v>1</v>
+      </c>
       <c r="I16" s="1"/>
       <c r="K16" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="L16" s="6">
         <f>SUMIFS(D:D,G:G,"X")</f>
-        <v>0</v>
-      </c>
-      <c r="M16" s="7" t="e">
+        <v>3.7</v>
+      </c>
+      <c r="M16" s="7">
         <f>L16/SUM($L$15:$L$18)</f>
-        <v>#DIV/0!</v>
+        <v>0.46250000000000002</v>
       </c>
     </row>
     <row r="17" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="16"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="4"/>
+      <c r="A17" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" s="4">
+        <v>1</v>
+      </c>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="1"/>
+      <c r="G17" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H17" s="1">
+        <v>1</v>
+      </c>
       <c r="I17" s="1"/>
-      <c r="K17" t="s">
-        <v>10</v>
-      </c>
-      <c r="L17" s="6">
-        <f>SUMIFS(E:E,G:G,"X")</f>
-        <v>0</v>
-      </c>
-      <c r="M17" s="7" t="e">
-        <f>L17/SUM($L$15:$L$18)</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="K18" t="s">
-        <v>13</v>
-      </c>
-      <c r="L18" s="6">
-        <f>SUMIFS(F:F,G:G,"X")</f>
-        <v>0</v>
-      </c>
-      <c r="M18" s="7" t="e">
-        <f>L18/SUM($L$15:$L$18)</f>
-        <v>#DIV/0!</v>
-      </c>
+    </row>
+    <row r="18" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+    </row>
+    <row r="19" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
     </row>
     <row r="20" spans="1:15" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="K20" s="10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" s="4">
+        <v>1</v>
+      </c>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="K20" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C21" s="4">
+        <v>1</v>
+      </c>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
       <c r="L21" s="19" t="s">
         <v>4</v>
       </c>
@@ -1385,8 +1753,9 @@
       <c r="O21" s="19"/>
     </row>
     <row r="22" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="K22" s="11" t="s">
-        <v>26</v>
+      <c r="G22"/>
+      <c r="K22" s="10" t="s">
+        <v>22</v>
       </c>
       <c r="L22">
         <v>1</v>
@@ -1402,126 +1771,109 @@
       </c>
     </row>
     <row r="23" spans="1:15" ht="127.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K23" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="L23" s="12" t="s">
-        <v>40</v>
-      </c>
+      <c r="G23"/>
+      <c r="K23" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L23" s="11"/>
       <c r="M23" s="8"/>
       <c r="N23" s="8"/>
       <c r="O23" s="8"/>
     </row>
     <row r="24" spans="1:15" ht="123.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K24" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="L24" s="12" t="s">
-        <v>27</v>
-      </c>
+      <c r="K24" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="L24" s="11"/>
       <c r="M24" s="8"/>
       <c r="N24" s="8"/>
       <c r="O24" s="8"/>
     </row>
-    <row r="25" spans="1:15" ht="117.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K25" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="L25" s="8"/>
-      <c r="M25" s="8"/>
-      <c r="N25" s="8"/>
-      <c r="O25" s="8"/>
-    </row>
-    <row r="26" spans="1:15" ht="101.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K26" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="L26" s="9"/>
-      <c r="M26" s="9"/>
-      <c r="N26" s="9"/>
-      <c r="O26" s="9"/>
+    <row r="25" spans="1:15" ht="57" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:15" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K26" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K27" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="L27" s="20"/>
+      <c r="M27" s="21"/>
+      <c r="N27" s="21"/>
+      <c r="O27" s="22"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K28" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="L28" s="20"/>
+      <c r="M28" s="21"/>
+      <c r="N28" s="21"/>
+      <c r="O28" s="22"/>
     </row>
     <row r="30" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="K30" s="11" t="s">
+      <c r="K30" s="10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" ht="44.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K31" s="12" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="31" spans="1:15" ht="44.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K31" s="13" t="s">
+      <c r="L31" s="20"/>
+      <c r="M31" s="21"/>
+      <c r="N31" s="21"/>
+      <c r="O31" s="22"/>
+    </row>
+    <row r="32" spans="1:15" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K32" s="12" t="s">
         <v>29</v>
-      </c>
-      <c r="L31" s="20"/>
-      <c r="M31" s="20"/>
-      <c r="N31" s="20"/>
-      <c r="O31" s="20"/>
-    </row>
-    <row r="32" spans="1:15" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K32" s="13" t="s">
-        <v>30</v>
       </c>
       <c r="L32" s="17"/>
       <c r="M32" s="17"/>
       <c r="N32" s="17"/>
       <c r="O32" s="17"/>
     </row>
-    <row r="34" spans="11:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="K34" s="11" t="s">
+    <row r="33" spans="11:15" x14ac:dyDescent="0.25">
+      <c r="K33" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="L33" s="17"/>
+      <c r="M33" s="17"/>
+      <c r="N33" s="17"/>
+      <c r="O33" s="17"/>
+    </row>
+    <row r="34" spans="11:15" x14ac:dyDescent="0.25">
+      <c r="K34" s="12"/>
+      <c r="L34" s="12"/>
+      <c r="M34" s="12"/>
+      <c r="N34" s="12"/>
+      <c r="O34" s="12"/>
+    </row>
+    <row r="35" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K35" s="12" t="s">
         <v>31</v>
-      </c>
-    </row>
-    <row r="35" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K35" s="13" t="s">
-        <v>32</v>
       </c>
       <c r="L35" s="17"/>
       <c r="M35" s="17"/>
       <c r="N35" s="17"/>
       <c r="O35" s="17"/>
     </row>
-    <row r="36" spans="11:15" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K36" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="L36" s="17"/>
-      <c r="M36" s="17"/>
-      <c r="N36" s="17"/>
-      <c r="O36" s="17"/>
-    </row>
-    <row r="37" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K37" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="L37" s="17"/>
-      <c r="M37" s="17"/>
-      <c r="N37" s="17"/>
-      <c r="O37" s="17"/>
-    </row>
-    <row r="38" spans="11:15" x14ac:dyDescent="0.25">
-      <c r="K38" s="13"/>
-      <c r="L38" s="13"/>
-      <c r="M38" s="13"/>
-      <c r="N38" s="13"/>
-      <c r="O38" s="13"/>
-    </row>
-    <row r="39" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K39" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="L39" s="17"/>
-      <c r="M39" s="17"/>
-      <c r="N39" s="17"/>
-      <c r="O39" s="17"/>
-    </row>
+    <row r="36" spans="11:15" ht="30.6" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="L32:O32"/>
+    <mergeCell ref="L33:O33"/>
     <mergeCell ref="L35:O35"/>
-    <mergeCell ref="L36:O36"/>
-    <mergeCell ref="L37:O37"/>
-    <mergeCell ref="L39:O39"/>
     <mergeCell ref="B1:I1"/>
     <mergeCell ref="L21:O21"/>
     <mergeCell ref="L31:O31"/>
-    <mergeCell ref="L32:O32"/>
+    <mergeCell ref="L27:O27"/>
+    <mergeCell ref="L28:O28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
@@ -1560,17 +1912,17 @@
       <c r="G1" s="18"/>
       <c r="H1" s="18"/>
       <c r="I1" s="18"/>
-      <c r="K1" s="10" t="s">
+      <c r="K1" s="9" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="K2" t="s">
-        <v>14</v>
-      </c>
-      <c r="L2" s="6" t="e">
+        <v>10</v>
+      </c>
+      <c r="L2" s="6">
         <f>AVERAGEIFS(H:H,G:G, "X", B:B, "Récit")</f>
-        <v>#DIV/0!</v>
+        <v>2.3333333333333335</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -1578,19 +1930,19 @@
         <v>0</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>1</v>
@@ -1602,19 +1954,19 @@
         <v>6</v>
       </c>
       <c r="K3" t="s">
-        <v>15</v>
-      </c>
-      <c r="L3" s="6" t="e">
+        <v>11</v>
+      </c>
+      <c r="L3" s="6">
         <f>AVERAGEIFS(H:H,G:G, "X", B:B, "Tâche")</f>
-        <v>#DIV/0!</v>
+        <v>1.6363636363636365</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
-        <v>44</v>
+      <c r="A4" s="23" t="s">
+        <v>48</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
@@ -1624,82 +1976,90 @@
       <c r="H4" s="5"/>
       <c r="I4" s="5"/>
       <c r="K4" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="L4" s="6">
         <f>COUNTIFS(G:G, "X", B:B, "Récit")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
-        <v>45</v>
+      <c r="A5" s="23" t="s">
+        <v>49</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
-      <c r="G5" s="3"/>
+      <c r="G5" s="3" t="s">
+        <v>58</v>
+      </c>
       <c r="H5" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I5" s="1"/>
       <c r="K5" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="L5" s="6">
         <f>COUNTIFS(G:G, "X", B:B, "Tâche")</f>
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
-        <v>46</v>
+      <c r="A6" s="23" t="s">
+        <v>59</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="4">
-        <v>0.1</v>
-      </c>
-      <c r="D6" s="4"/>
+        <v>9</v>
+      </c>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4">
+        <v>1</v>
+      </c>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
-      <c r="G6" s="3"/>
+      <c r="G6" s="3" t="s">
+        <v>58</v>
+      </c>
       <c r="H6" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I6" s="1"/>
     </row>
     <row r="7" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="16" t="s">
-        <v>49</v>
+      <c r="A7" s="23" t="s">
+        <v>60</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
+      <c r="D7" s="4">
+        <v>1</v>
+      </c>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
-      <c r="G7" s="3"/>
+      <c r="G7" s="3" t="s">
+        <v>58</v>
+      </c>
       <c r="H7" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I7" s="1"/>
-      <c r="K7" s="11" t="s">
-        <v>24</v>
+      <c r="K7" s="10" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="16" t="s">
-        <v>47</v>
+      <c r="A8" s="23" t="s">
+        <v>61</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C8" s="4"/>
       <c r="D8" s="4">
@@ -1707,139 +2067,145 @@
       </c>
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
-      <c r="G8" s="3"/>
+      <c r="G8" s="3" t="s">
+        <v>58</v>
+      </c>
       <c r="H8" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I8" s="1"/>
       <c r="K8" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="L8" s="6">
         <f>COUNTIF(B:B,"Récit")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="16" t="s">
-        <v>48</v>
+      <c r="A9" s="14" t="s">
+        <v>73</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C9" s="4"/>
       <c r="D9" s="4">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
-      <c r="G9" s="3"/>
+      <c r="G9" s="3" t="s">
+        <v>58</v>
+      </c>
       <c r="H9" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I9" s="1"/>
       <c r="K9" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="L9" s="6">
         <f>COUNTIF(B:B, "Tâche")</f>
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="16" t="s">
-        <v>50</v>
+      <c r="A10" s="14" t="s">
+        <v>62</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="C10" s="4"/>
-      <c r="D10" s="4">
-        <v>1</v>
-      </c>
+      <c r="D10" s="4"/>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
       <c r="G10" s="3"/>
       <c r="H10" s="1"/>
-      <c r="I10" s="1">
-        <v>5</v>
-      </c>
+      <c r="I10" s="1"/>
     </row>
     <row r="11" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="16" t="s">
-        <v>54</v>
+      <c r="A11" s="14" t="s">
+        <v>63</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C11" s="4">
-        <v>0.45</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="C11" s="4"/>
       <c r="D11" s="4"/>
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1">
-        <v>4</v>
-      </c>
+      <c r="G11" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H11" s="1">
+        <v>3</v>
+      </c>
+      <c r="I11" s="1"/>
       <c r="K11" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="L11" s="7">
         <f>L4/L8</f>
-        <v>0</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="16" t="s">
-        <v>51</v>
+      <c r="A12" s="14" t="s">
+        <v>64</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12" s="4"/>
+        <v>9</v>
+      </c>
+      <c r="C12" s="4">
+        <v>1</v>
+      </c>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
-      <c r="G12" s="3"/>
+      <c r="G12" s="3" t="s">
+        <v>58</v>
+      </c>
       <c r="H12" s="1">
         <v>2</v>
       </c>
       <c r="I12" s="1"/>
       <c r="K12" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L12" s="7">
         <f>L5/L9</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="16" t="s">
-        <v>52</v>
+      <c r="A13" s="14" t="s">
+        <v>65</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C13" s="4">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
-      <c r="G13" s="3"/>
+      <c r="G13" s="3" t="s">
+        <v>58</v>
+      </c>
       <c r="H13" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I13" s="1"/>
     </row>
     <row r="14" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="16" t="s">
-        <v>53</v>
+      <c r="A14" s="14" t="s">
+        <v>66</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C14" s="4">
         <v>1</v>
@@ -1847,42 +2213,58 @@
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
-      <c r="G14" s="3"/>
+      <c r="G14" s="3" t="s">
+        <v>58</v>
+      </c>
       <c r="H14" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I14" s="1"/>
-      <c r="K14" s="11" t="s">
-        <v>22</v>
+      <c r="K14" s="10" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="16"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
+      <c r="A15" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="D15" s="4">
+        <v>0.5</v>
+      </c>
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="1"/>
+      <c r="G15" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H15" s="1">
+        <v>3</v>
+      </c>
       <c r="I15" s="1"/>
       <c r="K15" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="L15" s="6">
         <f>SUMIFS(C:C,G:G,"X")</f>
-        <v>0</v>
-      </c>
-      <c r="M15" s="7" t="e">
+        <v>6.5</v>
+      </c>
+      <c r="M15" s="7">
         <f>L15/SUM($L$15:$L$18)</f>
-        <v>#DIV/0!</v>
+        <v>0.59090909090909094</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="B16" s="3"/>
+      <c r="A16" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
@@ -1891,58 +2273,114 @@
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
       <c r="K16" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="L16" s="6">
         <f>SUMIFS(D:D,G:G,"X")</f>
-        <v>0</v>
-      </c>
-      <c r="M16" s="7" t="e">
+        <v>4.5</v>
+      </c>
+      <c r="M16" s="7">
         <f>L16/SUM($L$15:$L$18)</f>
-        <v>#DIV/0!</v>
+        <v>0.40909090909090912</v>
       </c>
     </row>
     <row r="17" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="16"/>
-      <c r="B17" s="3"/>
+      <c r="A17" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>8</v>
+      </c>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
       <c r="G17" s="3"/>
-      <c r="H17" s="1"/>
+      <c r="H17" s="1">
+        <v>1</v>
+      </c>
       <c r="I17" s="1"/>
-      <c r="K17" t="s">
-        <v>10</v>
-      </c>
-      <c r="L17" s="6">
-        <f>SUMIFS(E:E,G:G,"X")</f>
-        <v>0</v>
-      </c>
-      <c r="M17" s="7" t="e">
-        <f>L17/SUM($L$15:$L$18)</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="K18" t="s">
-        <v>13</v>
-      </c>
-      <c r="L18" s="6">
-        <f>SUMIFS(F:F,G:G,"X")</f>
-        <v>0</v>
-      </c>
-      <c r="M18" s="7" t="e">
-        <f>L18/SUM($L$15:$L$18)</f>
-        <v>#DIV/0!</v>
-      </c>
+    </row>
+    <row r="18" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" s="4">
+        <v>1</v>
+      </c>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H18" s="1">
+        <v>1</v>
+      </c>
+      <c r="I18" s="1"/>
+    </row>
+    <row r="19" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
     </row>
     <row r="20" spans="1:15" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="K20" s="10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H20" s="1">
+        <v>1</v>
+      </c>
+      <c r="I20" s="1"/>
+      <c r="K20" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C21" s="4">
+        <v>1</v>
+      </c>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H21" s="1">
+        <v>1</v>
+      </c>
+      <c r="I21" s="1">
+        <v>2</v>
+      </c>
       <c r="L21" s="19" t="s">
         <v>4</v>
       </c>
@@ -1950,9 +2388,30 @@
       <c r="N21" s="19"/>
       <c r="O21" s="19"/>
     </row>
-    <row r="22" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="K22" s="11" t="s">
-        <v>26</v>
+    <row r="22" spans="1:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" s="4">
+        <v>1</v>
+      </c>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H22" s="1">
+        <v>1</v>
+      </c>
+      <c r="I22" s="1">
+        <v>2</v>
+      </c>
+      <c r="K22" s="10" t="s">
+        <v>22</v>
       </c>
       <c r="L22">
         <v>1</v>
@@ -1968,126 +2427,727 @@
       </c>
     </row>
     <row r="23" spans="1:15" ht="127.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K23" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="L23" s="12" t="s">
-        <v>40</v>
+      <c r="K23" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="L23" s="11" t="s">
+        <v>34</v>
       </c>
       <c r="M23" s="8"/>
       <c r="N23" s="8"/>
       <c r="O23" s="8"/>
     </row>
     <row r="24" spans="1:15" ht="123.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K24" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="L24" s="12" t="s">
-        <v>27</v>
+      <c r="K24" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="L24" s="11" t="s">
+        <v>23</v>
       </c>
       <c r="M24" s="8"/>
       <c r="N24" s="8"/>
       <c r="O24" s="8"/>
     </row>
-    <row r="25" spans="1:15" ht="117.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K25" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="L25" s="8"/>
-      <c r="M25" s="8"/>
-      <c r="N25" s="8"/>
-      <c r="O25" s="8"/>
-    </row>
-    <row r="26" spans="1:15" ht="101.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K26" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="L26" s="9"/>
-      <c r="M26" s="9"/>
-      <c r="N26" s="9"/>
-      <c r="O26" s="9"/>
+    <row r="25" spans="1:15" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:15" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K26" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K27" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="L27" s="16"/>
+      <c r="M27" s="16"/>
+      <c r="N27" s="16"/>
+      <c r="O27" s="16"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K28" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="L28" s="15"/>
+      <c r="M28" s="15"/>
+      <c r="N28" s="15"/>
+      <c r="O28" s="15"/>
     </row>
     <row r="30" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="K30" s="11" t="s">
+      <c r="K30" s="10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" ht="44.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K31" s="12" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="31" spans="1:15" ht="44.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K31" s="13" t="s">
+      <c r="L31" s="15"/>
+      <c r="M31" s="15"/>
+      <c r="N31" s="15"/>
+      <c r="O31" s="15"/>
+    </row>
+    <row r="32" spans="1:15" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K32" s="12" t="s">
         <v>29</v>
-      </c>
-      <c r="L31" s="20"/>
-      <c r="M31" s="20"/>
-      <c r="N31" s="20"/>
-      <c r="O31" s="20"/>
-    </row>
-    <row r="32" spans="1:15" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K32" s="13" t="s">
-        <v>30</v>
       </c>
       <c r="L32" s="17"/>
       <c r="M32" s="17"/>
       <c r="N32" s="17"/>
       <c r="O32" s="17"/>
     </row>
-    <row r="34" spans="11:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="K34" s="11" t="s">
+    <row r="33" spans="11:15" x14ac:dyDescent="0.25">
+      <c r="K33" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="L33" s="17"/>
+      <c r="M33" s="17"/>
+      <c r="N33" s="17"/>
+      <c r="O33" s="17"/>
+    </row>
+    <row r="34" spans="11:15" x14ac:dyDescent="0.25">
+      <c r="K34" s="12"/>
+      <c r="L34" s="12"/>
+      <c r="M34" s="12"/>
+      <c r="N34" s="12"/>
+      <c r="O34" s="12"/>
+    </row>
+    <row r="35" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K35" s="12" t="s">
         <v>31</v>
-      </c>
-    </row>
-    <row r="35" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K35" s="13" t="s">
-        <v>32</v>
       </c>
       <c r="L35" s="17"/>
       <c r="M35" s="17"/>
       <c r="N35" s="17"/>
       <c r="O35" s="17"/>
     </row>
-    <row r="36" spans="11:15" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K36" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="L36" s="17"/>
-      <c r="M36" s="17"/>
-      <c r="N36" s="17"/>
-      <c r="O36" s="17"/>
-    </row>
-    <row r="37" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K37" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="L37" s="17"/>
-      <c r="M37" s="17"/>
-      <c r="N37" s="17"/>
-      <c r="O37" s="17"/>
-    </row>
-    <row r="38" spans="11:15" x14ac:dyDescent="0.25">
-      <c r="K38" s="13"/>
-      <c r="L38" s="13"/>
-      <c r="M38" s="13"/>
-      <c r="N38" s="13"/>
-      <c r="O38" s="13"/>
-    </row>
-    <row r="39" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K39" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="L39" s="17"/>
-      <c r="M39" s="17"/>
-      <c r="N39" s="17"/>
-      <c r="O39" s="17"/>
-    </row>
+    <row r="36" spans="11:15" ht="30.6" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="L37:O37"/>
-    <mergeCell ref="L39:O39"/>
+  <mergeCells count="5">
+    <mergeCell ref="L33:O33"/>
+    <mergeCell ref="L35:O35"/>
     <mergeCell ref="B1:I1"/>
     <mergeCell ref="L21:O21"/>
-    <mergeCell ref="L31:O31"/>
     <mergeCell ref="L32:O32"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6A37C47-DF27-4421-A54B-1AE7B0D5C7F9}">
+  <dimension ref="A1:O39"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="66.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="6" width="10.28515625" customWidth="1"/>
+    <col min="7" max="7" width="8.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.42578125" customWidth="1"/>
+    <col min="11" max="11" width="47.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="30" customWidth="1"/>
+    <col min="13" max="14" width="26.7109375" customWidth="1"/>
+    <col min="15" max="15" width="29.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" ht="18" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="K1" s="9" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="K2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L2" s="6">
+        <f>AVERAGEIFS(H:H,G:G, "X", B:B, "Récit")</f>
+        <v>2.3333333333333335</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="K3" t="s">
+        <v>11</v>
+      </c>
+      <c r="L3" s="6">
+        <f>AVERAGEIFS(H:H,G:G, "X", B:B, "Tâche")</f>
+        <v>1.6363636363636365</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="23"/>
+      <c r="B4" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="K4" t="s">
+        <v>16</v>
+      </c>
+      <c r="L4" s="6">
+        <f>COUNTIFS(G:G, "X", B:B, "Récit")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="23"/>
+      <c r="B5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H5" s="1">
+        <v>3</v>
+      </c>
+      <c r="I5" s="1"/>
+      <c r="K5" t="s">
+        <v>17</v>
+      </c>
+      <c r="L5" s="6">
+        <f>COUNTIFS(G:G, "X", B:B, "Tâche")</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="23"/>
+      <c r="B6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4">
+        <v>1</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" s="1">
+        <v>2</v>
+      </c>
+      <c r="I6" s="1"/>
+    </row>
+    <row r="7" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="23"/>
+      <c r="B7" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4">
+        <v>1</v>
+      </c>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H7" s="1">
+        <v>1</v>
+      </c>
+      <c r="I7" s="1"/>
+      <c r="K7" s="10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="23"/>
+      <c r="B8" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4">
+        <v>1</v>
+      </c>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H8" s="1">
+        <v>3</v>
+      </c>
+      <c r="I8" s="1"/>
+      <c r="K8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L8" s="6">
+        <f>COUNTIF(B:B,"Récit")</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="14"/>
+      <c r="B9" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4">
+        <v>1</v>
+      </c>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H9" s="1">
+        <v>2</v>
+      </c>
+      <c r="I9" s="1"/>
+      <c r="K9" t="s">
+        <v>14</v>
+      </c>
+      <c r="L9" s="6">
+        <f>COUNTIF(B:B, "Tâche")</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="14"/>
+      <c r="B10" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+    </row>
+    <row r="11" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="14"/>
+      <c r="B11" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H11" s="1">
+        <v>3</v>
+      </c>
+      <c r="I11" s="1"/>
+      <c r="K11" t="s">
+        <v>12</v>
+      </c>
+      <c r="L11" s="7">
+        <f>L4/L8</f>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="14"/>
+      <c r="B12" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="4">
+        <v>1</v>
+      </c>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H12" s="1">
+        <v>2</v>
+      </c>
+      <c r="I12" s="1"/>
+      <c r="K12" t="s">
+        <v>15</v>
+      </c>
+      <c r="L12" s="7">
+        <f>L5/L9</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="14"/>
+      <c r="B13" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="4">
+        <v>1</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H13" s="1">
+        <v>1</v>
+      </c>
+      <c r="I13" s="1"/>
+    </row>
+    <row r="14" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="14"/>
+      <c r="B14" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="4">
+        <v>1</v>
+      </c>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H14" s="1">
+        <v>1</v>
+      </c>
+      <c r="I14" s="1"/>
+      <c r="K14" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="14"/>
+      <c r="B15" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="D15" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H15" s="1">
+        <v>3</v>
+      </c>
+      <c r="I15" s="1"/>
+      <c r="K15" t="s">
+        <v>35</v>
+      </c>
+      <c r="L15" s="6">
+        <f>SUMIFS(C:C,G:G,"X")</f>
+        <v>6.5</v>
+      </c>
+      <c r="M15" s="7">
+        <f>L15/SUM($L$15:$L$18)</f>
+        <v>0.59090909090909094</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="14"/>
+      <c r="B16" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="K16" t="s">
+        <v>36</v>
+      </c>
+      <c r="L16" s="6">
+        <f>SUMIFS(D:D,G:G,"X")</f>
+        <v>4.5</v>
+      </c>
+      <c r="M16" s="7">
+        <f>L16/SUM($L$15:$L$18)</f>
+        <v>0.40909090909090912</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="14"/>
+      <c r="B17" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="1">
+        <v>1</v>
+      </c>
+      <c r="I17" s="1"/>
+    </row>
+    <row r="18" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="13"/>
+      <c r="B18" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" s="4">
+        <v>1</v>
+      </c>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H18" s="1">
+        <v>1</v>
+      </c>
+      <c r="I18" s="1"/>
+    </row>
+    <row r="19" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="14"/>
+      <c r="B19" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+    </row>
+    <row r="20" spans="1:15" ht="18" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="14"/>
+      <c r="B20" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H20" s="1">
+        <v>1</v>
+      </c>
+      <c r="I20" s="1"/>
+      <c r="K20" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="14"/>
+      <c r="B21" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C21" s="4">
+        <v>1</v>
+      </c>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H21" s="1">
+        <v>1</v>
+      </c>
+      <c r="I21" s="1">
+        <v>2</v>
+      </c>
+      <c r="L21" s="19" t="s">
+        <v>4</v>
+      </c>
+      <c r="M21" s="19"/>
+      <c r="N21" s="19"/>
+      <c r="O21" s="19"/>
+    </row>
+    <row r="22" spans="1:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="14"/>
+      <c r="B22" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" s="4">
+        <v>1</v>
+      </c>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H22" s="1">
+        <v>1</v>
+      </c>
+      <c r="I22" s="1">
+        <v>2</v>
+      </c>
+      <c r="K22" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="L22">
+        <v>1</v>
+      </c>
+      <c r="M22">
+        <v>2</v>
+      </c>
+      <c r="N22">
+        <v>3</v>
+      </c>
+      <c r="O22">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" ht="127.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K23" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="L23" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="M23" s="8"/>
+      <c r="N23" s="8"/>
+      <c r="O23" s="8"/>
+    </row>
+    <row r="24" spans="1:15" ht="123.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K24" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="L24" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="M24" s="8"/>
+      <c r="N24" s="8"/>
+      <c r="O24" s="8"/>
+    </row>
+    <row r="25" spans="1:15" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:15" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K26" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K27" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="L27" s="16"/>
+      <c r="M27" s="16"/>
+      <c r="N27" s="16"/>
+      <c r="O27" s="16"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K28" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="L28" s="15"/>
+      <c r="M28" s="15"/>
+      <c r="N28" s="15"/>
+      <c r="O28" s="15"/>
+    </row>
+    <row r="30" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K30" s="10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" ht="44.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K31" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="L31" s="15"/>
+      <c r="M31" s="15"/>
+      <c r="N31" s="15"/>
+      <c r="O31" s="15"/>
+    </row>
+    <row r="32" spans="1:15" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K32" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="L32" s="17"/>
+      <c r="M32" s="17"/>
+      <c r="N32" s="17"/>
+      <c r="O32" s="17"/>
+    </row>
+    <row r="33" spans="11:15" x14ac:dyDescent="0.25">
+      <c r="K33" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="L33" s="17"/>
+      <c r="M33" s="17"/>
+      <c r="N33" s="17"/>
+      <c r="O33" s="17"/>
+    </row>
+    <row r="34" spans="11:15" x14ac:dyDescent="0.25">
+      <c r="K34" s="12"/>
+      <c r="L34" s="12"/>
+      <c r="M34" s="12"/>
+      <c r="N34" s="12"/>
+      <c r="O34" s="12"/>
+    </row>
+    <row r="35" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K35" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="L35" s="17"/>
+      <c r="M35" s="17"/>
+      <c r="N35" s="17"/>
+      <c r="O35" s="17"/>
+    </row>
+    <row r="36" spans="11:15" ht="30.6" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B1:I1"/>
+    <mergeCell ref="L21:O21"/>
+    <mergeCell ref="L32:O32"/>
+    <mergeCell ref="L33:O33"/>
     <mergeCell ref="L35:O35"/>
-    <mergeCell ref="L36:O36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>

</xml_diff>

<commit_message>
Update journal de sprint
</commit_message>
<xml_diff>
--- a/Journal_de_sprint.xlsx
+++ b/Journal_de_sprint.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2281126\Documents\GitHub\projet-de-session-5gd-a25-gr-e\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4280962-EBDA-4371-8521-508C8F5F891F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{391F71FE-0CEC-486C-99B2-0FD82349CFF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{6BF6013A-4C68-4CEF-BF49-8F7071437FDB}"/>
+    <workbookView xWindow="14295" yWindow="660" windowWidth="14610" windowHeight="14925" xr2:uid="{6BF6013A-4C68-4CEF-BF49-8F7071437FDB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint1" sheetId="1" r:id="rId1"/>
@@ -303,7 +303,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="93">
   <si>
     <t>Item planifié</t>
   </si>
@@ -401,12 +401,6 @@
     <t>Bilan de la mesure d'amélioration du sprint courant</t>
   </si>
   <si>
-    <t>Membre 1</t>
-  </si>
-  <si>
-    <t>Membre 2</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -771,6 +765,445 @@
   </si>
   <si>
     <t>Avoir un style de compteur de pièces plus ambiant</t>
+  </si>
+  <si>
+    <t>ABSCENT (pew pew)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Progrès accomplis:  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Soumettre un request au prof pour l'installation de Unity 2022.3.17f1 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">                       Objectifs pour la journée : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Créer projet Unity 3D                           </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Obstacles rencontrés: I</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">l manque le install 2022.3.17f1                                         </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Actions Suivantes:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> aide de l'enseignant.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Progrès accomplis:  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Création du répo git et du projet Unity     </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Objectifs pour la journée : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Créer projet Unity 3D                           </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Obstacles rencontrés: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">                       </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Actions Suivantes:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> map</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Progrès accomplis:  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Soumettre un request au prof pour l'installation de Unity 2022.3.17f1 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">                          Objectifs pour la journée : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Map                           </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Obstacles rencontrés: I</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">l manque toujours le install 2022.3.17f1                                         </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Actions Suivantes:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> attendre que le technicien installe Unity</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Progrès accomplis:  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Unity Baseline                 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">                  Objectifs pour la journée : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Map                           </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Obstacles rencontrés: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">               </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Actions Suivantes:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> attendre que le technicien installe Unity</t>
+    </r>
+  </si>
+  <si>
+    <t>Absent (il manque toujours la bonne version de Unity)</t>
+  </si>
+  <si>
+    <t>abscent</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Progrès accomplis:  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>basic UI</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">           Objectifs pour la journée : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">basic UI                           </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Obstacles rencontrés: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Transformer projet 2022.3.17f1 en 6000                                                              </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Actions Suivantes:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> attendre</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -963,7 +1396,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="3"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -980,14 +1413,8 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="4"/>
     <xf numFmtId="9" fontId="4" fillId="3" borderId="3" xfId="4" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="3" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="2"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="3" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -1000,6 +1427,22 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="3" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="3" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="3" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -1015,15 +1458,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -1382,17 +1816,17 @@
       <c r="A1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="K1" s="9" t="s">
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="K1" s="8" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1413,16 +1847,16 @@
         <v>19</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>37</v>
-      </c>
       <c r="F3" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>1</v>
@@ -1442,11 +1876,11 @@
       </c>
     </row>
     <row r="4" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
-        <v>41</v>
+      <c r="A4" s="12" t="s">
+        <v>39</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
@@ -1464,8 +1898,8 @@
       </c>
     </row>
     <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="14" t="s">
-        <v>42</v>
+      <c r="A5" s="12" t="s">
+        <v>40</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>8</v>
@@ -1475,7 +1909,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H5" s="1">
         <v>1</v>
@@ -1490,8 +1924,8 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
-        <v>57</v>
+      <c r="A6" s="12" t="s">
+        <v>55</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>9</v>
@@ -1503,7 +1937,7 @@
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
       <c r="G6" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H6" s="1">
         <v>1</v>
@@ -1511,8 +1945,8 @@
       <c r="I6" s="1"/>
     </row>
     <row r="7" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="14" t="s">
-        <v>52</v>
+      <c r="A7" s="12" t="s">
+        <v>50</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>9</v>
@@ -1526,19 +1960,19 @@
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H7" s="1">
         <v>1</v>
       </c>
       <c r="I7" s="1"/>
-      <c r="K7" s="10" t="s">
+      <c r="K7" s="9" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
-        <v>53</v>
+      <c r="A8" s="12" t="s">
+        <v>51</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>9</v>
@@ -1552,7 +1986,7 @@
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="G8" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H8" s="1">
         <v>1</v>
@@ -1567,11 +2001,11 @@
       </c>
     </row>
     <row r="9" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="14" t="s">
-        <v>43</v>
+      <c r="A9" s="12" t="s">
+        <v>41</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -1589,8 +2023,8 @@
       </c>
     </row>
     <row r="10" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
-        <v>45</v>
+      <c r="A10" s="12" t="s">
+        <v>43</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>8</v>
@@ -1600,7 +2034,7 @@
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
       <c r="G10" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H10" s="1">
         <v>2</v>
@@ -1608,8 +2042,8 @@
       <c r="I10" s="1"/>
     </row>
     <row r="11" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
-        <v>50</v>
+      <c r="A11" s="12" t="s">
+        <v>48</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>9</v>
@@ -1621,7 +2055,7 @@
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
       <c r="G11" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H11" s="1">
         <v>1</v>
@@ -1636,8 +2070,8 @@
       </c>
     </row>
     <row r="12" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="14" t="s">
-        <v>51</v>
+      <c r="A12" s="12" t="s">
+        <v>49</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>9</v>
@@ -1649,7 +2083,7 @@
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
       <c r="G12" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H12" s="1">
         <v>2</v>
@@ -1664,11 +2098,11 @@
       </c>
     </row>
     <row r="13" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="14" t="s">
-        <v>46</v>
+      <c r="A13" s="12" t="s">
+        <v>44</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -1679,8 +2113,8 @@
       <c r="I13" s="1"/>
     </row>
     <row r="14" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="14" t="s">
-        <v>47</v>
+      <c r="A14" s="12" t="s">
+        <v>45</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>8</v>
@@ -1690,19 +2124,19 @@
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
       <c r="G14" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H14" s="1">
         <v>1</v>
       </c>
       <c r="I14" s="1"/>
-      <c r="K14" s="10" t="s">
+      <c r="K14" s="9" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="14" t="s">
-        <v>54</v>
+      <c r="A15" s="12" t="s">
+        <v>52</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>9</v>
@@ -1714,14 +2148,14 @@
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
       <c r="G15" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H15" s="1">
         <v>1</v>
       </c>
       <c r="I15" s="1"/>
       <c r="K15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="L15" s="6">
         <f>SUMIFS(C:C,G:G,"X")</f>
@@ -1733,8 +2167,8 @@
       </c>
     </row>
     <row r="16" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="14" t="s">
-        <v>56</v>
+      <c r="A16" s="12" t="s">
+        <v>54</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>9</v>
@@ -1746,14 +2180,14 @@
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
       <c r="G16" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H16" s="1">
         <v>1</v>
       </c>
       <c r="I16" s="1"/>
       <c r="K16" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L16" s="6">
         <f>SUMIFS(D:D,G:G,"X")</f>
@@ -1765,8 +2199,8 @@
       </c>
     </row>
     <row r="17" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="14" t="s">
-        <v>55</v>
+      <c r="A17" s="12" t="s">
+        <v>53</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>9</v>
@@ -1778,7 +2212,7 @@
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
       <c r="G17" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H17" s="1">
         <v>1</v>
@@ -1786,11 +2220,11 @@
       <c r="I17" s="1"/>
     </row>
     <row r="18" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="14" t="s">
-        <v>71</v>
+      <c r="A18" s="12" t="s">
+        <v>69</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -1801,8 +2235,8 @@
       <c r="I18" s="1"/>
     </row>
     <row r="19" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="14" t="s">
-        <v>72</v>
+      <c r="A19" s="12" t="s">
+        <v>70</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>8</v>
@@ -1816,8 +2250,8 @@
       <c r="I19" s="1"/>
     </row>
     <row r="20" spans="1:15" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="14" t="s">
-        <v>38</v>
+      <c r="A20" s="12" t="s">
+        <v>36</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>9</v>
@@ -1831,13 +2265,13 @@
       <c r="G20" s="3"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
-      <c r="K20" s="9" t="s">
+      <c r="K20" s="8" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="21" spans="1:15" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="14" t="s">
-        <v>39</v>
+      <c r="A21" s="12" t="s">
+        <v>37</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>9</v>
@@ -1851,121 +2285,137 @@
       <c r="G21" s="3"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
-      <c r="L21" s="20" t="s">
+      <c r="L21" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="M21" s="20"/>
-      <c r="N21" s="20"/>
-      <c r="O21" s="20"/>
+      <c r="M21" s="24"/>
+      <c r="N21" s="24"/>
+      <c r="O21" s="24"/>
     </row>
     <row r="22" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="G22"/>
-      <c r="K22" s="10" t="s">
+      <c r="K22" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="L22">
-        <v>1</v>
-      </c>
-      <c r="M22">
-        <v>2</v>
-      </c>
-      <c r="N22">
-        <v>3</v>
-      </c>
-      <c r="O22">
-        <v>4</v>
+      <c r="L22" s="21">
+        <v>45903</v>
+      </c>
+      <c r="M22" s="21">
+        <v>45905</v>
+      </c>
+      <c r="N22" s="21">
+        <v>45910</v>
+      </c>
+      <c r="O22" s="21">
+        <v>45912</v>
       </c>
     </row>
     <row r="23" spans="1:15" ht="127.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="G23"/>
-      <c r="K23" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="L23" s="11"/>
-      <c r="M23" s="8"/>
-      <c r="N23" s="8"/>
-      <c r="O23" s="8"/>
+      <c r="K23" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="L23" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="M23" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="N23" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="O23" s="19" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="24" spans="1:15" ht="123.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K24" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="L24" s="11"/>
-      <c r="M24" s="8"/>
-      <c r="N24" s="8"/>
-      <c r="O24" s="8"/>
+      <c r="K24" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="L24" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="M24" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="N24" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="O24" s="19" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="25" spans="1:15" ht="57" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:15" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="K26" s="10" t="s">
+      <c r="K26" s="9" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="K27" s="12" t="s">
+      <c r="K27" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="L27" s="21"/>
-      <c r="M27" s="22"/>
-      <c r="N27" s="22"/>
-      <c r="O27" s="23"/>
+      <c r="L27" s="25"/>
+      <c r="M27" s="26"/>
+      <c r="N27" s="26"/>
+      <c r="O27" s="27"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="K28" s="12" t="s">
+      <c r="K28" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="L28" s="21"/>
-      <c r="M28" s="22"/>
-      <c r="N28" s="22"/>
-      <c r="O28" s="23"/>
+      <c r="L28" s="25"/>
+      <c r="M28" s="26"/>
+      <c r="N28" s="26"/>
+      <c r="O28" s="27"/>
     </row>
     <row r="30" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="K30" s="10" t="s">
+      <c r="K30" s="9" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="31" spans="1:15" ht="44.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K31" s="12" t="s">
+      <c r="K31" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="L31" s="21"/>
-      <c r="M31" s="22"/>
-      <c r="N31" s="22"/>
-      <c r="O31" s="23"/>
+      <c r="L31" s="25"/>
+      <c r="M31" s="26"/>
+      <c r="N31" s="26"/>
+      <c r="O31" s="27"/>
     </row>
     <row r="32" spans="1:15" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K32" s="12" t="s">
+      <c r="K32" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="L32" s="18"/>
-      <c r="M32" s="18"/>
-      <c r="N32" s="18"/>
-      <c r="O32" s="18"/>
+      <c r="L32" s="22"/>
+      <c r="M32" s="22"/>
+      <c r="N32" s="22"/>
+      <c r="O32" s="22"/>
     </row>
     <row r="33" spans="11:15" x14ac:dyDescent="0.25">
-      <c r="K33" s="12" t="s">
+      <c r="K33" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="L33" s="18"/>
-      <c r="M33" s="18"/>
-      <c r="N33" s="18"/>
-      <c r="O33" s="18"/>
+      <c r="L33" s="22"/>
+      <c r="M33" s="22"/>
+      <c r="N33" s="22"/>
+      <c r="O33" s="22"/>
     </row>
     <row r="34" spans="11:15" x14ac:dyDescent="0.25">
-      <c r="K34" s="12"/>
-      <c r="L34" s="12"/>
-      <c r="M34" s="12"/>
-      <c r="N34" s="12"/>
-      <c r="O34" s="12"/>
+      <c r="K34" s="10"/>
+      <c r="L34" s="10"/>
+      <c r="M34" s="10"/>
+      <c r="N34" s="10"/>
+      <c r="O34" s="10"/>
     </row>
     <row r="35" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K35" s="12" t="s">
+      <c r="K35" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="L35" s="18"/>
-      <c r="M35" s="18"/>
-      <c r="N35" s="18"/>
-      <c r="O35" s="18"/>
+      <c r="L35" s="22"/>
+      <c r="M35" s="22"/>
+      <c r="N35" s="22"/>
+      <c r="O35" s="22"/>
     </row>
     <row r="36" spans="11:15" ht="30.6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="37" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2008,17 +2458,17 @@
       <c r="A1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="K1" s="9" t="s">
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="K1" s="8" t="s">
         <v>3</v>
       </c>
     </row>
@@ -2039,16 +2489,16 @@
         <v>19</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>37</v>
-      </c>
       <c r="F3" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>1</v>
@@ -2068,11 +2518,11 @@
       </c>
     </row>
     <row r="4" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="17" t="s">
-        <v>48</v>
+      <c r="A4" s="15" t="s">
+        <v>46</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
@@ -2090,8 +2540,8 @@
       </c>
     </row>
     <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
-        <v>49</v>
+      <c r="A5" s="15" t="s">
+        <v>47</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>8</v>
@@ -2101,7 +2551,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H5" s="1">
         <v>3</v>
@@ -2116,8 +2566,8 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="17" t="s">
-        <v>59</v>
+      <c r="A6" s="15" t="s">
+        <v>57</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>9</v>
@@ -2129,7 +2579,7 @@
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
       <c r="G6" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H6" s="1">
         <v>2</v>
@@ -2137,8 +2587,8 @@
       <c r="I6" s="1"/>
     </row>
     <row r="7" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="17" t="s">
-        <v>60</v>
+      <c r="A7" s="15" t="s">
+        <v>58</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>9</v>
@@ -2150,19 +2600,19 @@
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H7" s="1">
         <v>1</v>
       </c>
       <c r="I7" s="1"/>
-      <c r="K7" s="10" t="s">
+      <c r="K7" s="9" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="17" t="s">
-        <v>61</v>
+      <c r="A8" s="15" t="s">
+        <v>59</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>9</v>
@@ -2174,7 +2624,7 @@
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="G8" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H8" s="1">
         <v>3</v>
@@ -2189,8 +2639,8 @@
       </c>
     </row>
     <row r="9" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="14" t="s">
-        <v>73</v>
+      <c r="A9" s="12" t="s">
+        <v>71</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>9</v>
@@ -2202,7 +2652,7 @@
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H9" s="1">
         <v>2</v>
@@ -2217,11 +2667,11 @@
       </c>
     </row>
     <row r="10" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
-        <v>62</v>
+      <c r="A10" s="12" t="s">
+        <v>60</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -2232,8 +2682,8 @@
       <c r="I10" s="1"/>
     </row>
     <row r="11" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
-        <v>63</v>
+      <c r="A11" s="12" t="s">
+        <v>61</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>8</v>
@@ -2243,7 +2693,7 @@
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
       <c r="G11" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H11" s="1">
         <v>3</v>
@@ -2258,8 +2708,8 @@
       </c>
     </row>
     <row r="12" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="14" t="s">
-        <v>64</v>
+      <c r="A12" s="12" t="s">
+        <v>62</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>9</v>
@@ -2271,7 +2721,7 @@
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
       <c r="G12" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H12" s="1">
         <v>2</v>
@@ -2286,8 +2736,8 @@
       </c>
     </row>
     <row r="13" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="14" t="s">
-        <v>65</v>
+      <c r="A13" s="12" t="s">
+        <v>63</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>9</v>
@@ -2299,7 +2749,7 @@
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
       <c r="G13" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H13" s="1">
         <v>1</v>
@@ -2307,8 +2757,8 @@
       <c r="I13" s="1"/>
     </row>
     <row r="14" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="14" t="s">
-        <v>66</v>
+      <c r="A14" s="12" t="s">
+        <v>64</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>9</v>
@@ -2320,19 +2770,19 @@
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
       <c r="G14" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H14" s="1">
         <v>1</v>
       </c>
       <c r="I14" s="1"/>
-      <c r="K14" s="10" t="s">
+      <c r="K14" s="9" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="14" t="s">
-        <v>67</v>
+      <c r="A15" s="12" t="s">
+        <v>65</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>9</v>
@@ -2346,14 +2796,14 @@
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
       <c r="G15" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H15" s="1">
         <v>3</v>
       </c>
       <c r="I15" s="1"/>
       <c r="K15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="L15" s="6">
         <f>SUMIFS(C:C,G:G,"X")</f>
@@ -2365,11 +2815,11 @@
       </c>
     </row>
     <row r="16" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="14" t="s">
-        <v>68</v>
+      <c r="A16" s="12" t="s">
+        <v>66</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
@@ -2379,7 +2829,7 @@
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
       <c r="K16" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L16" s="6">
         <f>SUMIFS(D:D,G:G,"X")</f>
@@ -2391,8 +2841,8 @@
       </c>
     </row>
     <row r="17" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="14" t="s">
-        <v>69</v>
+      <c r="A17" s="12" t="s">
+        <v>67</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>8</v>
@@ -2408,8 +2858,8 @@
       <c r="I17" s="1"/>
     </row>
     <row r="18" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="13" t="s">
-        <v>70</v>
+      <c r="A18" s="11" t="s">
+        <v>68</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>9</v>
@@ -2421,7 +2871,7 @@
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
       <c r="G18" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H18" s="1">
         <v>1</v>
@@ -2429,11 +2879,11 @@
       <c r="I18" s="1"/>
     </row>
     <row r="19" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="14" t="s">
-        <v>71</v>
+      <c r="A19" s="12" t="s">
+        <v>69</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -2444,8 +2894,8 @@
       <c r="I19" s="1"/>
     </row>
     <row r="20" spans="1:15" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="14" t="s">
-        <v>72</v>
+      <c r="A20" s="12" t="s">
+        <v>70</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>8</v>
@@ -2455,19 +2905,19 @@
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
       <c r="G20" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H20" s="1">
         <v>1</v>
       </c>
       <c r="I20" s="1"/>
-      <c r="K20" s="9" t="s">
+      <c r="K20" s="8" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="21" spans="1:15" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="14" t="s">
-        <v>38</v>
+      <c r="A21" s="12" t="s">
+        <v>36</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>9</v>
@@ -2479,7 +2929,7 @@
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
       <c r="G21" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H21" s="1">
         <v>1</v>
@@ -2487,16 +2937,16 @@
       <c r="I21" s="1">
         <v>2</v>
       </c>
-      <c r="L21" s="20" t="s">
+      <c r="L21" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="M21" s="20"/>
-      <c r="N21" s="20"/>
-      <c r="O21" s="20"/>
+      <c r="M21" s="24"/>
+      <c r="N21" s="24"/>
+      <c r="O21" s="24"/>
     </row>
     <row r="22" spans="1:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="14" t="s">
-        <v>39</v>
+      <c r="A22" s="12" t="s">
+        <v>37</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>9</v>
@@ -2508,7 +2958,7 @@
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
       <c r="G22" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H22" s="1">
         <v>1</v>
@@ -2516,115 +2966,117 @@
       <c r="I22" s="1">
         <v>2</v>
       </c>
-      <c r="K22" s="10" t="s">
+      <c r="K22" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="L22">
-        <v>1</v>
-      </c>
-      <c r="M22">
-        <v>2</v>
-      </c>
-      <c r="N22">
-        <v>3</v>
-      </c>
-      <c r="O22">
-        <v>4</v>
+      <c r="L22" s="21">
+        <v>45917</v>
+      </c>
+      <c r="M22" s="21">
+        <v>45919</v>
+      </c>
+      <c r="N22" s="21">
+        <v>45924</v>
+      </c>
+      <c r="O22" s="21">
+        <v>45926</v>
       </c>
     </row>
     <row r="23" spans="1:15" ht="127.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K23" s="12" t="s">
+      <c r="K23" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="L23" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="L23" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="M23" s="8"/>
-      <c r="N23" s="8"/>
-      <c r="O23" s="8"/>
+      <c r="M23" s="20"/>
+      <c r="N23" s="20"/>
+      <c r="O23" s="20"/>
     </row>
     <row r="24" spans="1:15" ht="123.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K24" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="L24" s="11" t="s">
+      <c r="K24" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="L24" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="M24" s="8"/>
-      <c r="N24" s="8"/>
-      <c r="O24" s="8"/>
+      <c r="M24" s="20"/>
+      <c r="N24" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="O24" s="20"/>
     </row>
     <row r="25" spans="1:15" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:15" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="K26" s="10" t="s">
+      <c r="K26" s="9" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="K27" s="12" t="s">
+      <c r="K27" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="L27" s="16"/>
-      <c r="M27" s="16"/>
-      <c r="N27" s="16"/>
-      <c r="O27" s="16"/>
+      <c r="L27" s="14"/>
+      <c r="M27" s="14"/>
+      <c r="N27" s="14"/>
+      <c r="O27" s="14"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="K28" s="12" t="s">
+      <c r="K28" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="L28" s="15"/>
-      <c r="M28" s="15"/>
-      <c r="N28" s="15"/>
-      <c r="O28" s="15"/>
+      <c r="L28" s="13"/>
+      <c r="M28" s="13"/>
+      <c r="N28" s="13"/>
+      <c r="O28" s="13"/>
     </row>
     <row r="30" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="K30" s="10" t="s">
+      <c r="K30" s="9" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="31" spans="1:15" ht="44.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K31" s="12" t="s">
+      <c r="K31" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="L31" s="15"/>
-      <c r="M31" s="15"/>
-      <c r="N31" s="15"/>
-      <c r="O31" s="15"/>
+      <c r="L31" s="13"/>
+      <c r="M31" s="13"/>
+      <c r="N31" s="13"/>
+      <c r="O31" s="13"/>
     </row>
     <row r="32" spans="1:15" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K32" s="12" t="s">
+      <c r="K32" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="L32" s="18"/>
-      <c r="M32" s="18"/>
-      <c r="N32" s="18"/>
-      <c r="O32" s="18"/>
+      <c r="L32" s="22"/>
+      <c r="M32" s="22"/>
+      <c r="N32" s="22"/>
+      <c r="O32" s="22"/>
     </row>
     <row r="33" spans="11:15" x14ac:dyDescent="0.25">
-      <c r="K33" s="12" t="s">
+      <c r="K33" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="L33" s="18"/>
-      <c r="M33" s="18"/>
-      <c r="N33" s="18"/>
-      <c r="O33" s="18"/>
+      <c r="L33" s="22"/>
+      <c r="M33" s="22"/>
+      <c r="N33" s="22"/>
+      <c r="O33" s="22"/>
     </row>
     <row r="34" spans="11:15" x14ac:dyDescent="0.25">
-      <c r="K34" s="12"/>
-      <c r="L34" s="12"/>
-      <c r="M34" s="12"/>
-      <c r="N34" s="12"/>
-      <c r="O34" s="12"/>
+      <c r="K34" s="10"/>
+      <c r="L34" s="10"/>
+      <c r="M34" s="10"/>
+      <c r="N34" s="10"/>
+      <c r="O34" s="10"/>
     </row>
     <row r="35" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K35" s="12" t="s">
+      <c r="K35" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="L35" s="18"/>
-      <c r="M35" s="18"/>
-      <c r="N35" s="18"/>
-      <c r="O35" s="18"/>
+      <c r="L35" s="22"/>
+      <c r="M35" s="22"/>
+      <c r="N35" s="22"/>
+      <c r="O35" s="22"/>
     </row>
     <row r="36" spans="11:15" ht="30.6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="37" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2664,17 +3116,17 @@
       <c r="A1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="K1" s="9" t="s">
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="K1" s="8" t="s">
         <v>3</v>
       </c>
     </row>
@@ -2695,10 +3147,10 @@
         <v>19</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
@@ -2720,9 +3172,9 @@
       </c>
     </row>
     <row r="4" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="17"/>
+      <c r="A4" s="15"/>
       <c r="B4" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
@@ -2740,7 +3192,7 @@
       </c>
     </row>
     <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="17"/>
+      <c r="A5" s="15"/>
       <c r="B5" s="3" t="s">
         <v>8</v>
       </c>
@@ -2749,7 +3201,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
@@ -2762,7 +3214,7 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="17"/>
+      <c r="A6" s="15"/>
       <c r="B6" s="3" t="s">
         <v>9</v>
       </c>
@@ -2773,13 +3225,13 @@
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
       <c r="G6" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
     </row>
     <row r="7" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="17"/>
+      <c r="A7" s="15"/>
       <c r="B7" s="3" t="s">
         <v>9</v>
       </c>
@@ -2790,16 +3242,16 @@
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
-      <c r="K7" s="10" t="s">
+      <c r="K7" s="9" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="17"/>
+      <c r="A8" s="15"/>
       <c r="B8" s="3" t="s">
         <v>9</v>
       </c>
@@ -2810,7 +3262,7 @@
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="G8" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
@@ -2823,7 +3275,7 @@
       </c>
     </row>
     <row r="9" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="14"/>
+      <c r="A9" s="12"/>
       <c r="B9" s="3" t="s">
         <v>9</v>
       </c>
@@ -2834,7 +3286,7 @@
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
@@ -2847,9 +3299,9 @@
       </c>
     </row>
     <row r="10" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="14"/>
+      <c r="A10" s="12"/>
       <c r="B10" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -2860,7 +3312,7 @@
       <c r="I10" s="1"/>
     </row>
     <row r="11" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="14"/>
+      <c r="A11" s="12"/>
       <c r="B11" s="3" t="s">
         <v>8</v>
       </c>
@@ -2880,8 +3332,8 @@
       </c>
     </row>
     <row r="12" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="14" t="s">
-        <v>85</v>
+      <c r="A12" s="12" t="s">
+        <v>83</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>9</v>
@@ -2902,8 +3354,8 @@
       </c>
     </row>
     <row r="13" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="14" t="s">
-        <v>86</v>
+      <c r="A13" s="12" t="s">
+        <v>84</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>9</v>
@@ -2917,8 +3369,8 @@
       <c r="I13" s="1"/>
     </row>
     <row r="14" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="14" t="s">
-        <v>83</v>
+      <c r="A14" s="12" t="s">
+        <v>81</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>9</v>
@@ -2930,19 +3382,19 @@
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
       <c r="G14" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H14" s="1">
         <v>1</v>
       </c>
       <c r="I14" s="1"/>
-      <c r="K14" s="10" t="s">
+      <c r="K14" s="9" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="14" t="s">
-        <v>84</v>
+      <c r="A15" s="12" t="s">
+        <v>82</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>9</v>
@@ -2954,14 +3406,14 @@
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
       <c r="G15" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H15" s="1">
         <v>1</v>
       </c>
       <c r="I15" s="1"/>
       <c r="K15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="L15" s="6">
         <f>SUMIFS(C:C,G:G,"X")</f>
@@ -2973,11 +3425,11 @@
       </c>
     </row>
     <row r="16" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="14" t="s">
-        <v>68</v>
+      <c r="A16" s="12" t="s">
+        <v>66</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
@@ -2987,7 +3439,7 @@
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
       <c r="K16" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L16" s="6">
         <f>SUMIFS(D:D,G:G,"X")</f>
@@ -2999,8 +3451,8 @@
       </c>
     </row>
     <row r="17" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="14" t="s">
-        <v>81</v>
+      <c r="A17" s="12" t="s">
+        <v>79</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>8</v>
@@ -3016,8 +3468,8 @@
       <c r="I17" s="1"/>
     </row>
     <row r="18" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="13" t="s">
-        <v>82</v>
+      <c r="A18" s="11" t="s">
+        <v>80</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>9</v>
@@ -3029,7 +3481,7 @@
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
       <c r="G18" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H18" s="1">
         <v>1</v>
@@ -3037,11 +3489,11 @@
       <c r="I18" s="1"/>
     </row>
     <row r="19" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="14" t="s">
-        <v>71</v>
+      <c r="A19" s="12" t="s">
+        <v>69</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -3052,8 +3504,8 @@
       <c r="I19" s="1"/>
     </row>
     <row r="20" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="14" t="s">
-        <v>72</v>
+      <c r="A20" s="12" t="s">
+        <v>70</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>8</v>
@@ -3063,7 +3515,7 @@
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
       <c r="G20" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H20" s="1">
         <v>1</v>
@@ -3071,7 +3523,7 @@
       <c r="I20" s="1"/>
     </row>
     <row r="21" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="14"/>
+      <c r="A21" s="12"/>
       <c r="B21" s="3"/>
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
@@ -3082,11 +3534,11 @@
       <c r="I21" s="1"/>
     </row>
     <row r="22" spans="1:15" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="14" t="s">
-        <v>77</v>
+      <c r="A22" s="12" t="s">
+        <v>75</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
@@ -3097,8 +3549,8 @@
       <c r="I22" s="1"/>
     </row>
     <row r="23" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="14" t="s">
-        <v>78</v>
+      <c r="A23" s="12" t="s">
+        <v>76</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>8</v>
@@ -3112,8 +3564,8 @@
       <c r="I23" s="1"/>
     </row>
     <row r="24" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="14" t="s">
-        <v>79</v>
+      <c r="A24" s="12" t="s">
+        <v>77</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>9</v>
@@ -3125,7 +3577,7 @@
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
       <c r="G24" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H24" s="1">
         <v>1</v>
@@ -3133,8 +3585,8 @@
       <c r="I24" s="1"/>
     </row>
     <row r="25" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="14" t="s">
-        <v>80</v>
+      <c r="A25" s="12" t="s">
+        <v>78</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>9</v>
@@ -3146,7 +3598,7 @@
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
       <c r="G25" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H25" s="1">
         <v>1</v>
@@ -3155,127 +3607,131 @@
     </row>
     <row r="26" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="27" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="14"/>
+      <c r="A27" s="12"/>
     </row>
     <row r="28" spans="1:15" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="K28" s="9" t="s">
+      <c r="K28" s="8" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="29" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="L29" s="20" t="s">
+      <c r="L29" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="M29" s="20"/>
-      <c r="N29" s="20"/>
-      <c r="O29" s="20"/>
+      <c r="M29" s="24"/>
+      <c r="N29" s="24"/>
+      <c r="O29" s="24"/>
     </row>
     <row r="30" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="K30" s="10" t="s">
+      <c r="K30" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="L30">
-        <v>1</v>
-      </c>
-      <c r="M30">
-        <v>2</v>
-      </c>
-      <c r="N30">
-        <v>3</v>
-      </c>
-      <c r="O30">
-        <v>4</v>
+      <c r="L30" s="21">
+        <v>45931</v>
+      </c>
+      <c r="M30" s="21">
+        <v>45933</v>
+      </c>
+      <c r="N30" s="21">
+        <v>45938</v>
+      </c>
+      <c r="O30" s="21">
+        <v>45940</v>
       </c>
     </row>
     <row r="31" spans="1:15" ht="44.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K31" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="L31" s="11"/>
-      <c r="M31" s="8"/>
-      <c r="N31" s="8"/>
-      <c r="O31" s="8"/>
+      <c r="K31" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="L31" s="19"/>
+      <c r="M31" s="20"/>
+      <c r="N31" s="20"/>
+      <c r="O31" s="20"/>
     </row>
     <row r="32" spans="1:15" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K32" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="L32" s="11"/>
-      <c r="M32" s="8"/>
-      <c r="N32" s="8"/>
-      <c r="O32" s="8"/>
+      <c r="K32" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="L32" s="19"/>
+      <c r="M32" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="N32" s="20"/>
+      <c r="O32" s="20" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="34" spans="11:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="K34" s="10" t="s">
+      <c r="K34" s="9" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="35" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K35" s="12" t="s">
+      <c r="K35" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="L35" s="16"/>
-      <c r="M35" s="16"/>
-      <c r="N35" s="16"/>
-      <c r="O35" s="16"/>
+      <c r="L35" s="14"/>
+      <c r="M35" s="14"/>
+      <c r="N35" s="14"/>
+      <c r="O35" s="14"/>
     </row>
     <row r="36" spans="11:15" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K36" s="12" t="s">
+      <c r="K36" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="L36" s="15"/>
-      <c r="M36" s="15"/>
-      <c r="N36" s="15"/>
-      <c r="O36" s="15"/>
+      <c r="L36" s="13"/>
+      <c r="M36" s="13"/>
+      <c r="N36" s="13"/>
+      <c r="O36" s="13"/>
     </row>
     <row r="37" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="38" spans="11:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="K38" s="10" t="s">
+      <c r="K38" s="9" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="39" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K39" s="12" t="s">
+      <c r="K39" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="L39" s="15"/>
-      <c r="M39" s="15"/>
-      <c r="N39" s="15"/>
-      <c r="O39" s="15"/>
+      <c r="L39" s="13"/>
+      <c r="M39" s="13"/>
+      <c r="N39" s="13"/>
+      <c r="O39" s="13"/>
     </row>
     <row r="40" spans="11:15" x14ac:dyDescent="0.25">
-      <c r="K40" s="12" t="s">
+      <c r="K40" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="L40" s="24"/>
-      <c r="M40" s="25"/>
-      <c r="N40" s="25"/>
-      <c r="O40" s="26"/>
+      <c r="L40" s="16"/>
+      <c r="M40" s="17"/>
+      <c r="N40" s="17"/>
+      <c r="O40" s="18"/>
     </row>
     <row r="41" spans="11:15" x14ac:dyDescent="0.25">
-      <c r="K41" s="12" t="s">
+      <c r="K41" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="L41" s="24"/>
-      <c r="M41" s="25"/>
-      <c r="N41" s="25"/>
-      <c r="O41" s="26"/>
+      <c r="L41" s="16"/>
+      <c r="M41" s="17"/>
+      <c r="N41" s="17"/>
+      <c r="O41" s="18"/>
     </row>
     <row r="42" spans="11:15" x14ac:dyDescent="0.25">
-      <c r="K42" s="12"/>
-      <c r="L42" s="12"/>
-      <c r="M42" s="12"/>
-      <c r="N42" s="12"/>
-      <c r="O42" s="12"/>
+      <c r="K42" s="10"/>
+      <c r="L42" s="10"/>
+      <c r="M42" s="10"/>
+      <c r="N42" s="10"/>
+      <c r="O42" s="10"/>
     </row>
     <row r="43" spans="11:15" x14ac:dyDescent="0.25">
-      <c r="K43" s="12" t="s">
+      <c r="K43" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="L43" s="24"/>
-      <c r="M43" s="25"/>
-      <c r="N43" s="25"/>
-      <c r="O43" s="26"/>
+      <c r="L43" s="16"/>
+      <c r="M43" s="17"/>
+      <c r="N43" s="17"/>
+      <c r="O43" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3309,17 +3765,17 @@
       <c r="A1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="K1" s="9" t="s">
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="K1" s="8" t="s">
         <v>3</v>
       </c>
     </row>
@@ -3340,16 +3796,16 @@
         <v>19</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>37</v>
-      </c>
       <c r="F3" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>1</v>
@@ -3369,9 +3825,9 @@
       </c>
     </row>
     <row r="4" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="17"/>
+      <c r="A4" s="15"/>
       <c r="B4" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
@@ -3389,7 +3845,7 @@
       </c>
     </row>
     <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="17"/>
+      <c r="A5" s="15"/>
       <c r="B5" s="3" t="s">
         <v>8</v>
       </c>
@@ -3398,7 +3854,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H5" s="1">
         <v>3</v>
@@ -3413,7 +3869,7 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="17"/>
+      <c r="A6" s="15"/>
       <c r="B6" s="3" t="s">
         <v>9</v>
       </c>
@@ -3424,7 +3880,7 @@
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
       <c r="G6" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H6" s="1">
         <v>2</v>
@@ -3432,7 +3888,7 @@
       <c r="I6" s="1"/>
     </row>
     <row r="7" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="17"/>
+      <c r="A7" s="15"/>
       <c r="B7" s="3" t="s">
         <v>9</v>
       </c>
@@ -3443,18 +3899,18 @@
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H7" s="1">
         <v>1</v>
       </c>
       <c r="I7" s="1"/>
-      <c r="K7" s="10" t="s">
+      <c r="K7" s="9" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="17"/>
+      <c r="A8" s="15"/>
       <c r="B8" s="3" t="s">
         <v>9</v>
       </c>
@@ -3465,7 +3921,7 @@
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="G8" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H8" s="1">
         <v>3</v>
@@ -3480,7 +3936,7 @@
       </c>
     </row>
     <row r="9" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="14"/>
+      <c r="A9" s="12"/>
       <c r="B9" s="3" t="s">
         <v>9</v>
       </c>
@@ -3491,7 +3947,7 @@
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H9" s="1">
         <v>2</v>
@@ -3506,9 +3962,9 @@
       </c>
     </row>
     <row r="10" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="14"/>
+      <c r="A10" s="12"/>
       <c r="B10" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -3519,7 +3975,7 @@
       <c r="I10" s="1"/>
     </row>
     <row r="11" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="14"/>
+      <c r="A11" s="12"/>
       <c r="B11" s="3" t="s">
         <v>8</v>
       </c>
@@ -3528,7 +3984,7 @@
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
       <c r="G11" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H11" s="1">
         <v>3</v>
@@ -3543,7 +3999,7 @@
       </c>
     </row>
     <row r="12" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="14"/>
+      <c r="A12" s="12"/>
       <c r="B12" s="3" t="s">
         <v>9</v>
       </c>
@@ -3554,7 +4010,7 @@
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
       <c r="G12" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H12" s="1">
         <v>2</v>
@@ -3569,7 +4025,7 @@
       </c>
     </row>
     <row r="13" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="14"/>
+      <c r="A13" s="12"/>
       <c r="B13" s="3" t="s">
         <v>9</v>
       </c>
@@ -3580,7 +4036,7 @@
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
       <c r="G13" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H13" s="1">
         <v>1</v>
@@ -3588,7 +4044,7 @@
       <c r="I13" s="1"/>
     </row>
     <row r="14" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="14"/>
+      <c r="A14" s="12"/>
       <c r="B14" s="3" t="s">
         <v>9</v>
       </c>
@@ -3599,18 +4055,18 @@
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
       <c r="G14" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H14" s="1">
         <v>1</v>
       </c>
       <c r="I14" s="1"/>
-      <c r="K14" s="10" t="s">
+      <c r="K14" s="9" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="14"/>
+      <c r="A15" s="12"/>
       <c r="B15" s="3" t="s">
         <v>9</v>
       </c>
@@ -3623,14 +4079,14 @@
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
       <c r="G15" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H15" s="1">
         <v>3</v>
       </c>
       <c r="I15" s="1"/>
       <c r="K15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="L15" s="6">
         <f>SUMIFS(C:C,G:G,"X")</f>
@@ -3642,9 +4098,9 @@
       </c>
     </row>
     <row r="16" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="14"/>
+      <c r="A16" s="12"/>
       <c r="B16" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
@@ -3654,7 +4110,7 @@
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
       <c r="K16" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="L16" s="6">
         <f>SUMIFS(D:D,G:G,"X")</f>
@@ -3666,7 +4122,7 @@
       </c>
     </row>
     <row r="17" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="14"/>
+      <c r="A17" s="12"/>
       <c r="B17" s="3" t="s">
         <v>8</v>
       </c>
@@ -3681,7 +4137,7 @@
       <c r="I17" s="1"/>
     </row>
     <row r="18" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="13"/>
+      <c r="A18" s="11"/>
       <c r="B18" s="3" t="s">
         <v>9</v>
       </c>
@@ -3692,7 +4148,7 @@
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
       <c r="G18" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H18" s="1">
         <v>1</v>
@@ -3700,9 +4156,9 @@
       <c r="I18" s="1"/>
     </row>
     <row r="19" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="14"/>
+      <c r="A19" s="12"/>
       <c r="B19" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -3713,7 +4169,7 @@
       <c r="I19" s="1"/>
     </row>
     <row r="20" spans="1:15" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="14"/>
+      <c r="A20" s="12"/>
       <c r="B20" s="3" t="s">
         <v>8</v>
       </c>
@@ -3722,18 +4178,18 @@
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
       <c r="G20" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H20" s="1">
         <v>1</v>
       </c>
       <c r="I20" s="1"/>
-      <c r="K20" s="9" t="s">
+      <c r="K20" s="8" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="21" spans="1:15" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="14"/>
+      <c r="A21" s="12"/>
       <c r="B21" s="3" t="s">
         <v>9</v>
       </c>
@@ -3744,7 +4200,7 @@
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
       <c r="G21" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H21" s="1">
         <v>1</v>
@@ -3752,15 +4208,15 @@
       <c r="I21" s="1">
         <v>2</v>
       </c>
-      <c r="L21" s="20" t="s">
+      <c r="L21" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="M21" s="20"/>
-      <c r="N21" s="20"/>
-      <c r="O21" s="20"/>
+      <c r="M21" s="24"/>
+      <c r="N21" s="24"/>
+      <c r="O21" s="24"/>
     </row>
     <row r="22" spans="1:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="14"/>
+      <c r="A22" s="12"/>
       <c r="B22" s="3" t="s">
         <v>9</v>
       </c>
@@ -3771,7 +4227,7 @@
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
       <c r="G22" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H22" s="1">
         <v>1</v>
@@ -3779,115 +4235,121 @@
       <c r="I22" s="1">
         <v>2</v>
       </c>
-      <c r="K22" s="10" t="s">
+      <c r="K22" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="L22">
-        <v>1</v>
-      </c>
-      <c r="M22">
-        <v>2</v>
-      </c>
-      <c r="N22">
-        <v>3</v>
-      </c>
-      <c r="O22">
-        <v>4</v>
+      <c r="L22" s="21">
+        <v>45947</v>
+      </c>
+      <c r="M22" s="21">
+        <v>45952</v>
+      </c>
+      <c r="N22" s="21">
+        <v>45954</v>
+      </c>
+      <c r="O22" s="21">
+        <v>45959</v>
       </c>
     </row>
     <row r="23" spans="1:15" ht="127.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K23" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="L23" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="M23" s="8"/>
-      <c r="N23" s="8"/>
-      <c r="O23" s="8"/>
+      <c r="K23" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="L23" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="M23" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="N23" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="O23" s="19" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="24" spans="1:15" ht="123.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K24" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="L24" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="M24" s="8"/>
-      <c r="N24" s="8"/>
-      <c r="O24" s="8"/>
+      <c r="K24" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="L24" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="M24" s="20"/>
+      <c r="N24" s="20"/>
+      <c r="O24" s="20"/>
     </row>
     <row r="25" spans="1:15" ht="56.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:15" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="K26" s="10" t="s">
+      <c r="K26" s="9" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="K27" s="12" t="s">
+      <c r="K27" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="L27" s="16"/>
-      <c r="M27" s="16"/>
-      <c r="N27" s="16"/>
-      <c r="O27" s="16"/>
+      <c r="L27" s="14"/>
+      <c r="M27" s="14"/>
+      <c r="N27" s="14"/>
+      <c r="O27" s="14"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="K28" s="12" t="s">
+      <c r="K28" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="L28" s="15"/>
-      <c r="M28" s="15"/>
-      <c r="N28" s="15"/>
-      <c r="O28" s="15"/>
+      <c r="L28" s="13"/>
+      <c r="M28" s="13"/>
+      <c r="N28" s="13"/>
+      <c r="O28" s="13"/>
     </row>
     <row r="30" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="K30" s="10" t="s">
+      <c r="K30" s="9" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="31" spans="1:15" ht="44.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K31" s="12" t="s">
+      <c r="K31" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="L31" s="15"/>
-      <c r="M31" s="15"/>
-      <c r="N31" s="15"/>
-      <c r="O31" s="15"/>
+      <c r="L31" s="13"/>
+      <c r="M31" s="13"/>
+      <c r="N31" s="13"/>
+      <c r="O31" s="13"/>
     </row>
     <row r="32" spans="1:15" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K32" s="12" t="s">
+      <c r="K32" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="L32" s="18"/>
-      <c r="M32" s="18"/>
-      <c r="N32" s="18"/>
-      <c r="O32" s="18"/>
+      <c r="L32" s="22"/>
+      <c r="M32" s="22"/>
+      <c r="N32" s="22"/>
+      <c r="O32" s="22"/>
     </row>
     <row r="33" spans="11:15" x14ac:dyDescent="0.25">
-      <c r="K33" s="12" t="s">
+      <c r="K33" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="L33" s="18"/>
-      <c r="M33" s="18"/>
-      <c r="N33" s="18"/>
-      <c r="O33" s="18"/>
+      <c r="L33" s="22"/>
+      <c r="M33" s="22"/>
+      <c r="N33" s="22"/>
+      <c r="O33" s="22"/>
     </row>
     <row r="34" spans="11:15" x14ac:dyDescent="0.25">
-      <c r="K34" s="12"/>
-      <c r="L34" s="12"/>
-      <c r="M34" s="12"/>
-      <c r="N34" s="12"/>
-      <c r="O34" s="12"/>
+      <c r="K34" s="10"/>
+      <c r="L34" s="10"/>
+      <c r="M34" s="10"/>
+      <c r="N34" s="10"/>
+      <c r="O34" s="10"/>
     </row>
     <row r="35" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K35" s="12" t="s">
+      <c r="K35" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="L35" s="18"/>
-      <c r="M35" s="18"/>
-      <c r="N35" s="18"/>
-      <c r="O35" s="18"/>
+      <c r="L35" s="22"/>
+      <c r="M35" s="22"/>
+      <c r="N35" s="22"/>
+      <c r="O35" s="22"/>
     </row>
     <row r="36" spans="11:15" ht="30.6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="37" spans="11:15" ht="31.15" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>